<commit_message>
updated l@age transition matrix, ran models
</commit_message>
<xml_diff>
--- a/Data/GOA_25.1.1_arrowtooth_single_species_1977-2024_new_data_clean_LA.xlsx
+++ b/Data/GOA_25.1.1_arrowtooth_single_species_1977-2024_new_data_clean_LA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kalei.shotwell\Work\GitHub\GOA-ATF-ESP\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05F69DA0-CC8B-4001-9D5D-A424D18BC998}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A7D86B-ED1C-4EF5-B970-DF4021EDB490}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data" sheetId="1" r:id="rId1"/>
@@ -76166,25 +76166,25 @@
         <v>1</v>
       </c>
       <c r="F2">
-        <v>0.99999999999807099</v>
+        <v>0.956955653525697</v>
       </c>
       <c r="G2">
-        <v>1.92845739377389E-12</v>
+        <v>4.2226794136929702E-2</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>8.1080075953744095E-4</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>6.7275561980652896E-6</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>2.3985037818583501E-8</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>3.6573393865286797E-11</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>2.64258626194269E-14</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -76534,43 +76534,43 @@
         <v>2</v>
       </c>
       <c r="F3">
-        <v>0.794698141222272</v>
+        <v>0.442724100919269</v>
       </c>
       <c r="G3">
-        <v>0.202477978920582</v>
+        <v>0.33657712513066901</v>
       </c>
       <c r="H3">
-        <v>2.8226551083182501E-3</v>
+        <v>0.16140992660911799</v>
       </c>
       <c r="I3">
-        <v>1.2247348540883601E-6</v>
+        <v>4.8797239546366E-2</v>
       </c>
       <c r="J3">
-        <v>1.39720457426051E-11</v>
+        <v>9.2910184596152294E-3</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>1.1127918506854599E-3</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>8.3726574749779905E-5</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>3.9518721541193002E-6</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>1.16850600799345E-7</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>2.1616031939288602E-9</v>
       </c>
       <c r="P3">
-        <v>0</v>
+        <v>2.49868375629472E-11</v>
       </c>
       <c r="Q3">
-        <v>0</v>
+        <v>1.8044452675657399E-13</v>
       </c>
       <c r="R3">
-        <v>0</v>
+        <v>7.2759889821199403E-16</v>
       </c>
       <c r="S3">
         <v>0</v>
@@ -76902,61 +76902,61 @@
         <v>3</v>
       </c>
       <c r="F4">
-        <v>4.60255797914663E-9</v>
+        <v>5.5409242140432198E-2</v>
       </c>
       <c r="G4">
-        <v>1.0318715363199301E-4</v>
+        <v>0.116627045554687</v>
       </c>
       <c r="H4">
-        <v>4.6630599205734598E-2</v>
+        <v>0.184335067112989</v>
       </c>
       <c r="I4">
-        <v>0.59246032972707596</v>
+        <v>0.21880088209670401</v>
       </c>
       <c r="J4">
-        <v>0.35238156073225102</v>
+        <v>0.195046471218144</v>
       </c>
       <c r="K4">
-        <v>8.4194669589040504E-3</v>
+        <v>0.13057638489895901</v>
       </c>
       <c r="L4">
-        <v>4.8515665750370397E-6</v>
+        <v>6.5643661125838901E-2</v>
       </c>
       <c r="M4">
-        <v>5.3268500721514998E-11</v>
+        <v>2.47777899989793E-2</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>7.0208898487675604E-3</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>1.49307261432549E-3</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>2.3823898405729601E-4</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>2.8514124666588801E-5</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>2.5590964242219802E-6</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>1.7216784895173301E-7</v>
       </c>
       <c r="T4">
-        <v>0</v>
+        <v>8.6798876922121504E-9</v>
       </c>
       <c r="U4">
-        <v>0</v>
+        <v>3.2781725100878797E-10</v>
       </c>
       <c r="V4">
-        <v>0</v>
+        <v>9.2718239105367803E-12</v>
       </c>
       <c r="W4">
-        <v>0</v>
+        <v>1.96322522186166E-13</v>
       </c>
       <c r="X4">
-        <v>0</v>
+        <v>3.1903834133561501E-15</v>
       </c>
       <c r="Y4">
         <v>0</v>
@@ -77270,82 +77270,82 @@
         <v>4</v>
       </c>
       <c r="F5">
-        <v>1.80141726837086E-25</v>
+        <v>5.4647242624280496E-3</v>
       </c>
       <c r="G5">
-        <v>7.9695485718750407E-18</v>
+        <v>1.5836476990310398E-2</v>
       </c>
       <c r="H5">
-        <v>1.22852777955677E-11</v>
+        <v>3.7794512653369E-2</v>
       </c>
       <c r="I5">
-        <v>6.7685338837152796E-7</v>
+        <v>7.4285046712054104E-2</v>
       </c>
       <c r="J5">
-        <v>1.4057209422319401E-3</v>
+        <v>0.120252614326691</v>
       </c>
       <c r="K5">
-        <v>0.12505495543492201</v>
+        <v>0.16033236250774199</v>
       </c>
       <c r="L5">
-        <v>0.63186546187229997</v>
+        <v>0.17607159264498801</v>
       </c>
       <c r="M5">
-        <v>0.236211491626584</v>
+        <v>0.15925805772415</v>
       </c>
       <c r="N5">
-        <v>5.4560087575249404E-3</v>
+        <v>0.11864646064017</v>
       </c>
       <c r="O5">
-        <v>5.6842727849115704E-6</v>
+        <v>7.2801668258574204E-2</v>
       </c>
       <c r="P5">
-        <v>2.27976526545603E-10</v>
+        <v>3.6791526519907497E-2</v>
       </c>
       <c r="Q5">
-        <v>3.3306690738754598E-16</v>
+        <v>1.5312850790798201E-2</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>5.2485977079669201E-3</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>1.48143470886754E-3</v>
       </c>
       <c r="T5">
-        <v>0</v>
+        <v>3.4430470260109197E-4</v>
       </c>
       <c r="U5">
-        <v>0</v>
+        <v>6.5885601284409399E-5</v>
       </c>
       <c r="V5">
-        <v>0</v>
+        <v>1.03797836816227E-5</v>
       </c>
       <c r="W5">
-        <v>0</v>
+        <v>1.3461614282268801E-6</v>
       </c>
       <c r="X5">
-        <v>0</v>
+        <v>1.4370638819595401E-7</v>
       </c>
       <c r="Y5">
-        <v>0</v>
+        <v>1.26264963177993E-8</v>
       </c>
       <c r="Z5">
-        <v>0</v>
+        <v>9.1300762463748799E-10</v>
       </c>
       <c r="AA5">
-        <v>0</v>
+        <v>5.43258957676455E-11</v>
       </c>
       <c r="AB5">
-        <v>0</v>
+        <v>2.6597382233748E-12</v>
       </c>
       <c r="AC5">
-        <v>0</v>
+        <v>1.07128190602281E-13</v>
       </c>
       <c r="AD5">
-        <v>0</v>
+        <v>3.5598152640425599E-15</v>
       </c>
       <c r="AE5">
-        <v>0</v>
+        <v>1.1124422700133E-16</v>
       </c>
       <c r="AF5">
         <v>0</v>
@@ -77638,91 +77638,91 @@
         <v>5</v>
       </c>
       <c r="F6">
-        <v>3.80597566990396E-31</v>
+        <v>4.3362137456427302E-4</v>
       </c>
       <c r="G6">
-        <v>2.53237626934299E-24</v>
+        <v>1.62017666538431E-3</v>
       </c>
       <c r="H6">
-        <v>2.1670489410149801E-18</v>
+        <v>5.1292922532595302E-3</v>
       </c>
       <c r="I6">
-        <v>2.4006045840733298E-13</v>
+        <v>1.3759846167465299E-2</v>
       </c>
       <c r="J6">
-        <v>3.4783000970005801E-9</v>
+        <v>3.1278530538445301E-2</v>
       </c>
       <c r="K6">
-        <v>6.7076396263007199E-6</v>
+        <v>6.0251657620809002E-2</v>
       </c>
       <c r="L6">
-        <v>1.77598655353646E-3</v>
+        <v>9.8354073372904305E-2</v>
       </c>
       <c r="M6">
-        <v>6.8269482507270995E-2</v>
+        <v>0.13605815963597601</v>
       </c>
       <c r="N6">
-        <v>0.41536936946724901</v>
+        <v>0.15950386447023199</v>
       </c>
       <c r="O6">
-        <v>0.43416571862367498</v>
+        <v>0.15846556692212099</v>
       </c>
       <c r="P6">
-        <v>7.8165190080339703E-2</v>
+        <v>0.133418353902855</v>
       </c>
       <c r="Q6">
-        <v>2.2381971506121299E-3</v>
+        <v>9.5194156733116597E-2</v>
       </c>
       <c r="R6">
-        <v>9.3391369548889696E-6</v>
+        <v>5.7559013790233898E-2</v>
       </c>
       <c r="S6">
-        <v>5.3617843498443496E-9</v>
+        <v>2.9492822144629199E-2</v>
       </c>
       <c r="T6">
-        <v>4.1022740759899499E-13</v>
+        <v>1.28058454138611E-2</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <v>4.7116786227236803E-3</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <v>1.4689357699546901E-3</v>
       </c>
       <c r="W6">
-        <v>0</v>
+        <v>3.88035852440976E-4</v>
       </c>
       <c r="X6">
-        <v>0</v>
+        <v>8.6848649758957297E-5</v>
       </c>
       <c r="Y6">
-        <v>0</v>
+        <v>1.6468538252781801E-5</v>
       </c>
       <c r="Z6">
-        <v>0</v>
+        <v>2.6456046849772399E-6</v>
       </c>
       <c r="AA6">
-        <v>0</v>
+        <v>3.60038298948937E-7</v>
       </c>
       <c r="AB6">
-        <v>0</v>
+        <v>4.1505079953692503E-8</v>
       </c>
       <c r="AC6">
-        <v>0</v>
+        <v>4.0528151125964103E-9</v>
       </c>
       <c r="AD6">
-        <v>0</v>
+        <v>3.3518838656107298E-10</v>
       </c>
       <c r="AE6">
-        <v>0</v>
+        <v>2.3478612140256201E-11</v>
       </c>
       <c r="AF6">
-        <v>0</v>
+        <v>1.39272092387945E-12</v>
       </c>
       <c r="AG6">
-        <v>0</v>
+        <v>5.7738569753433201E-14</v>
       </c>
       <c r="AH6">
-        <v>0</v>
+        <v>1.5322928126872699E-14</v>
       </c>
       <c r="AI6">
         <v>0</v>
@@ -78006,91 +78006,91 @@
         <v>6</v>
       </c>
       <c r="F7">
-        <v>6.8451730075273597E-50</v>
+        <v>1.02788890408052E-5</v>
       </c>
       <c r="G7">
-        <v>6.9474363936149102E-41</v>
+        <v>5.56573372089942E-5</v>
       </c>
       <c r="H7">
-        <v>8.3069432214695797E-33</v>
+        <v>2.5620077520497199E-4</v>
       </c>
       <c r="I7">
-        <v>1.17362658250122E-25</v>
+        <v>1.00262972798451E-3</v>
       </c>
       <c r="J7">
-        <v>1.96761608519514E-19</v>
+        <v>3.3359666065833401E-3</v>
       </c>
       <c r="K7">
-        <v>3.9394476624835397E-14</v>
+        <v>9.4371519954748705E-3</v>
       </c>
       <c r="L7">
-        <v>9.5143418106859793E-10</v>
+        <v>2.2699360080589301E-2</v>
       </c>
       <c r="M7">
-        <v>2.81927401327236E-6</v>
+        <v>4.6425105232825399E-2</v>
       </c>
       <c r="N7">
-        <v>1.05679696239839E-3</v>
+        <v>8.0736476157035705E-2</v>
       </c>
       <c r="O7">
-        <v>5.3017094309137001E-2</v>
+        <v>0.119391370169891</v>
       </c>
       <c r="P7">
-        <v>0.39021212192986898</v>
+        <v>0.15013035826370499</v>
       </c>
       <c r="Q7">
-        <v>0.46334765206074002</v>
+        <v>0.16053147497307099</v>
       </c>
       <c r="R7">
-        <v>8.9750691035236405E-2</v>
+        <v>0.14596510143566599</v>
       </c>
       <c r="S7">
-        <v>2.60256681826986E-3</v>
+        <v>0.11285830191261099</v>
       </c>
       <c r="T7">
-        <v>1.02515076512155E-5</v>
+        <v>7.4200961758546902E-2</v>
       </c>
       <c r="U7">
-        <v>5.1508913800901699E-9</v>
+        <v>4.14830312590828E-2</v>
       </c>
       <c r="V7">
-        <v>3.1896707497480702E-13</v>
+        <v>1.9720017726144401E-2</v>
       </c>
       <c r="W7">
-        <v>0</v>
+        <v>7.9709227263000393E-3</v>
       </c>
       <c r="X7">
-        <v>0</v>
+        <v>2.7394337279496102E-3</v>
       </c>
       <c r="Y7">
-        <v>0</v>
+        <v>8.0047594975972305E-4</v>
       </c>
       <c r="Z7">
-        <v>0</v>
+        <v>1.98862823218427E-4</v>
       </c>
       <c r="AA7">
-        <v>0</v>
+        <v>4.2000804123528802E-5</v>
       </c>
       <c r="AB7">
-        <v>0</v>
+        <v>7.5411869495999398E-6</v>
       </c>
       <c r="AC7">
-        <v>0</v>
+        <v>1.15100724001879E-6</v>
       </c>
       <c r="AD7">
-        <v>0</v>
+        <v>1.49330922795025E-7</v>
       </c>
       <c r="AE7">
-        <v>0</v>
+        <v>1.64676277397939E-8</v>
       </c>
       <c r="AF7">
-        <v>0</v>
+        <v>1.54346766519246E-9</v>
       </c>
       <c r="AG7">
-        <v>0</v>
+        <v>9.6977939153951305E-11</v>
       </c>
       <c r="AH7">
-        <v>0</v>
+        <v>3.47972297353024E-11</v>
       </c>
       <c r="AI7">
         <v>0</v>
@@ -78374,91 +78374,91 @@
         <v>7</v>
       </c>
       <c r="F8">
-        <v>1.17588351625797E-85</v>
+        <v>2.4507989475079498E-8</v>
       </c>
       <c r="G8">
-        <v>3.4259988580183401E-72</v>
+        <v>2.6118512132323E-7</v>
       </c>
       <c r="H8">
-        <v>6.6481233915814604E-60</v>
+        <v>2.2963073024727799E-6</v>
       </c>
       <c r="I8">
-        <v>8.6070937831010801E-49</v>
+        <v>1.6656847352866799E-5</v>
       </c>
       <c r="J8">
-        <v>7.4521045988196401E-39</v>
+        <v>9.9695568607539796E-5</v>
       </c>
       <c r="K8">
-        <v>4.3289667199007999E-30</v>
+        <v>4.9239806039138602E-4</v>
       </c>
       <c r="L8">
-        <v>1.6952136858000101E-22</v>
+        <v>2.00700796242221E-3</v>
       </c>
       <c r="M8">
-        <v>4.5073436778055496E-16</v>
+        <v>6.7515919163701702E-3</v>
       </c>
       <c r="N8">
-        <v>8.2325444636134405E-11</v>
+        <v>1.8746334668805702E-2</v>
       </c>
       <c r="O8">
-        <v>1.05434310379248E-6</v>
+        <v>4.2963997572285098E-2</v>
       </c>
       <c r="P8">
-        <v>9.8545192431339192E-4</v>
+        <v>8.1281564831464204E-2</v>
       </c>
       <c r="Q8">
-        <v>7.3126434683574104E-2</v>
+        <v>0.12693895869817801</v>
       </c>
       <c r="R8">
-        <v>0.50616787505014404</v>
+        <v>0.16365338911486901</v>
       </c>
       <c r="S8">
-        <v>0.38763802633882499</v>
+        <v>0.17417627951430301</v>
       </c>
       <c r="T8">
-        <v>3.18480818977721E-2</v>
+        <v>0.15303423966573099</v>
       </c>
       <c r="U8">
-        <v>2.32943989529554E-4</v>
+        <v>0.110999330720088</v>
       </c>
       <c r="V8">
-        <v>1.31685046089735E-7</v>
+        <v>6.6462361775605897E-2</v>
       </c>
       <c r="W8">
-        <v>5.3645976549887499E-12</v>
+        <v>3.2850459987399203E-2</v>
       </c>
       <c r="X8">
-        <v>0</v>
+        <v>1.34029182107697E-2</v>
       </c>
       <c r="Y8">
-        <v>0</v>
+        <v>4.5136419138174901E-3</v>
       </c>
       <c r="Z8">
-        <v>0</v>
+        <v>1.2545797232245599E-3</v>
       </c>
       <c r="AA8">
-        <v>0</v>
+        <v>2.8779476506353798E-4</v>
       </c>
       <c r="AB8">
-        <v>0</v>
+        <v>5.4481354687175201E-5</v>
       </c>
       <c r="AC8">
-        <v>0</v>
+        <v>8.5105487813942607E-6</v>
       </c>
       <c r="AD8">
-        <v>0</v>
+        <v>1.09691761973674E-6</v>
       </c>
       <c r="AE8">
-        <v>0</v>
+        <v>1.16642731487734E-7</v>
       </c>
       <c r="AF8">
-        <v>0</v>
+        <v>1.0232171242142599E-8</v>
       </c>
       <c r="AG8">
-        <v>0</v>
+        <v>5.9105387370854197E-10</v>
       </c>
       <c r="AH8">
-        <v>0</v>
+        <v>1.9579382599341699E-10</v>
       </c>
       <c r="AI8">
         <v>0</v>
@@ -78742,91 +78742,91 @@
         <v>8</v>
       </c>
       <c r="F9">
-        <v>1.71626190625254E-127</v>
+        <v>2.2927740517342199E-9</v>
       </c>
       <c r="G9">
-        <v>1.6344522506720799E-109</v>
+        <v>2.6113762780195501E-8</v>
       </c>
       <c r="H9">
-        <v>6.3820200183709502E-93</v>
+        <v>2.4949896231050502E-7</v>
       </c>
       <c r="I9">
-        <v>1.02293341024183E-77</v>
+        <v>1.9998165413849198E-6</v>
       </c>
       <c r="J9">
-        <v>6.7405628465405497E-64</v>
+        <v>1.3448192532881799E-5</v>
       </c>
       <c r="K9">
-        <v>1.8296869683820999E-51</v>
+        <v>7.5878573610330696E-5</v>
       </c>
       <c r="L9">
-        <v>2.05155375659752E-40</v>
+        <v>3.5923910704949201E-4</v>
       </c>
       <c r="M9">
-        <v>9.5391044203450006E-31</v>
+        <v>1.42719493398257E-3</v>
       </c>
       <c r="N9">
-        <v>1.84996137038377E-22</v>
+        <v>4.7581950356814298E-3</v>
       </c>
       <c r="O9">
-        <v>1.5100618697592199E-15</v>
+        <v>1.3313190807737799E-2</v>
       </c>
       <c r="P9">
-        <v>5.2685747493593703E-10</v>
+        <v>3.1262390184412098E-2</v>
       </c>
       <c r="Q9">
-        <v>8.0874302939979907E-6</v>
+        <v>6.1613886184652203E-2</v>
       </c>
       <c r="R9">
-        <v>5.8095695106428801E-3</v>
+        <v>0.101921229822363</v>
       </c>
       <c r="S9">
-        <v>0.225657569347541</v>
+        <v>0.14151103867130599</v>
       </c>
       <c r="T9">
-        <v>0.62281702758136503</v>
+        <v>0.16491576565374699</v>
       </c>
       <c r="U9">
-        <v>0.143480474151575</v>
+        <v>0.16131818134048201</v>
       </c>
       <c r="V9">
-        <v>2.2254699416263098E-3</v>
+        <v>0.132450407195915</v>
       </c>
       <c r="W9">
-        <v>1.80144288153272E-6</v>
+        <v>9.1278425365730401E-2</v>
       </c>
       <c r="X9">
-        <v>6.7213346000016801E-11</v>
+        <v>5.2798355063643103E-2</v>
       </c>
       <c r="Y9">
-        <v>1.11022302462515E-16</v>
+        <v>2.56329884849009E-2</v>
       </c>
       <c r="Z9">
-        <v>0</v>
+        <v>1.0444572489593599E-2</v>
       </c>
       <c r="AA9">
-        <v>0</v>
+        <v>3.57172191403942E-3</v>
       </c>
       <c r="AB9">
-        <v>0</v>
+        <v>1.0250388914224101E-3</v>
       </c>
       <c r="AC9">
-        <v>0</v>
+        <v>2.4686326026156501E-4</v>
       </c>
       <c r="AD9">
-        <v>0</v>
+        <v>4.9888613619854697E-5</v>
       </c>
       <c r="AE9">
-        <v>0</v>
+        <v>8.4595796282176405E-6</v>
       </c>
       <c r="AF9">
-        <v>0</v>
+        <v>1.2035673292387301E-6</v>
       </c>
       <c r="AG9">
-        <v>0</v>
+        <v>1.08263160678066E-7</v>
       </c>
       <c r="AH9">
-        <v>0</v>
+        <v>5.10811576462653E-8</v>
       </c>
       <c r="AI9">
         <v>0</v>
@@ -79110,91 +79110,91 @@
         <v>9</v>
       </c>
       <c r="F10">
-        <v>1.55522766799568E-137</v>
+        <v>1.1486265713567701E-11</v>
       </c>
       <c r="G10">
-        <v>8.5466260464286606E-120</v>
+        <v>1.99452895580657E-10</v>
       </c>
       <c r="H10">
-        <v>2.68864264084031E-103</v>
+        <v>2.8763217148463298E-9</v>
       </c>
       <c r="I10">
-        <v>4.8459455191943801E-88</v>
+        <v>3.44514712896393E-8</v>
       </c>
       <c r="J10">
-        <v>5.0095356088078504E-74</v>
+        <v>3.4275880199498999E-7</v>
       </c>
       <c r="K10">
-        <v>2.9743383538761701E-61</v>
+        <v>2.83280541955692E-6</v>
       </c>
       <c r="L10">
-        <v>1.0161273525764199E-49</v>
+        <v>1.9450375309606E-5</v>
       </c>
       <c r="M10">
-        <v>2.0023564423038E-39</v>
+        <v>1.10957549549647E-4</v>
       </c>
       <c r="N10">
-        <v>2.2838536894509901E-30</v>
+        <v>5.2593996218582495E-4</v>
       </c>
       <c r="O10">
-        <v>1.5153511379949699E-22</v>
+        <v>2.0715557861233401E-3</v>
       </c>
       <c r="P10">
-        <v>5.8942937034011798E-16</v>
+        <v>6.7805737327407698E-3</v>
       </c>
       <c r="Q10">
-        <v>1.36124856307821E-10</v>
+        <v>1.84446706211863E-2</v>
       </c>
       <c r="R10">
-        <v>1.9095411099924698E-6</v>
+        <v>4.1699616570262901E-2</v>
       </c>
       <c r="S10">
-        <v>1.7030322224921E-3</v>
+        <v>7.8355298635753995E-2</v>
       </c>
       <c r="T10">
-        <v>0.10665136361535101</v>
+        <v>0.122375480125406</v>
       </c>
       <c r="U10">
-        <v>0.56799276705229595</v>
+        <v>0.15886222776237</v>
       </c>
       <c r="V10">
-        <v>0.30788692975563098</v>
+        <v>0.17141676041048401</v>
       </c>
       <c r="W10">
-        <v>1.5703271222018599E-2</v>
+        <v>0.15374256670521799</v>
       </c>
       <c r="X10">
-        <v>6.0710982564660101E-5</v>
+        <v>0.11461476970406299</v>
       </c>
       <c r="Y10">
-        <v>1.5472165326713099E-8</v>
+        <v>7.1020822669870101E-2</v>
       </c>
       <c r="Z10">
-        <v>2.4358293160275899E-13</v>
+        <v>3.6577856483230899E-2</v>
       </c>
       <c r="AA10">
-        <v>0</v>
+        <v>1.5657519479361E-2</v>
       </c>
       <c r="AB10">
-        <v>0</v>
+        <v>5.5703272831156498E-3</v>
       </c>
       <c r="AC10">
-        <v>0</v>
+        <v>1.6469061845905701E-3</v>
       </c>
       <c r="AD10">
-        <v>0</v>
+        <v>4.04633242545814E-4</v>
       </c>
       <c r="AE10">
-        <v>0</v>
+        <v>8.2609527353552694E-5</v>
       </c>
       <c r="AF10">
-        <v>0</v>
+        <v>1.4013398953690801E-5</v>
       </c>
       <c r="AG10">
-        <v>0</v>
+        <v>1.45817110020014E-6</v>
       </c>
       <c r="AH10">
-        <v>0</v>
+        <v>7.7251627117513704E-7</v>
       </c>
       <c r="AI10">
         <v>0</v>
@@ -79478,91 +79478,91 @@
         <v>10</v>
       </c>
       <c r="F11">
-        <v>4.0967498325535001E-140</v>
+        <v>2.24241308564207E-10</v>
       </c>
       <c r="G11">
-        <v>2.7443182110807999E-123</v>
+        <v>2.1637871845160702E-9</v>
       </c>
       <c r="H11">
-        <v>1.48985569603171E-107</v>
+        <v>1.8254346765741601E-8</v>
       </c>
       <c r="I11">
-        <v>6.5592937568168098E-93</v>
+        <v>1.3464320493527699E-7</v>
       </c>
       <c r="J11">
-        <v>2.3438528886175199E-79</v>
+        <v>8.6832480843610403E-7</v>
       </c>
       <c r="K11">
-        <v>6.8047750110168005E-67</v>
+        <v>4.8963496412578004E-6</v>
       </c>
       <c r="L11">
-        <v>1.60725332614864E-55</v>
+        <v>2.41416757113003E-5</v>
       </c>
       <c r="M11">
-        <v>3.0938469946218398E-45</v>
+        <v>1.04082793226814E-4</v>
       </c>
       <c r="N11">
-        <v>4.8649281201011201E-36</v>
+        <v>3.9239016725970002E-4</v>
       </c>
       <c r="O11">
-        <v>6.26951698494494E-28</v>
+        <v>1.29358606960925E-3</v>
       </c>
       <c r="P11">
-        <v>6.6530484621587004E-21</v>
+        <v>3.7292385454726499E-3</v>
       </c>
       <c r="Q11">
-        <v>5.8552901095459401E-15</v>
+        <v>9.4015904351557305E-3</v>
       </c>
       <c r="R11">
-        <v>4.3236544479334402E-10</v>
+        <v>2.0727483921506799E-2</v>
       </c>
       <c r="S11">
-        <v>2.73365159758517E-6</v>
+        <v>3.9963425165677101E-2</v>
       </c>
       <c r="T11">
-        <v>1.5385321354870101E-3</v>
+        <v>6.7383781594933204E-2</v>
       </c>
       <c r="U11">
-        <v>8.3366534830105601E-2</v>
+        <v>9.9364033470090193E-2</v>
       </c>
       <c r="V11">
-        <v>0.49973771309436998</v>
+        <v>0.12814086483599901</v>
       </c>
       <c r="W11">
-        <v>0.37945426041636199</v>
+        <v>0.14452166957446799</v>
       </c>
       <c r="X11">
-        <v>3.5546880165235703E-2</v>
+        <v>0.14254968134243001</v>
       </c>
       <c r="Y11">
-        <v>3.5301660097020101E-4</v>
+        <v>0.122966657875517</v>
       </c>
       <c r="Z11">
-        <v>3.2864662224962802E-7</v>
+        <v>9.2767317718765396E-2</v>
       </c>
       <c r="AA11">
-        <v>2.68769451139405E-11</v>
+        <v>6.1204960674590497E-2</v>
       </c>
       <c r="AB11">
-        <v>2.2204460492503101E-16</v>
+        <v>3.53149465112719E-2</v>
       </c>
       <c r="AC11">
-        <v>0</v>
+        <v>1.7819928706281601E-2</v>
       </c>
       <c r="AD11">
-        <v>0</v>
+        <v>7.8636274047008594E-3</v>
       </c>
       <c r="AE11">
-        <v>0</v>
+        <v>3.03460714585752E-3</v>
       </c>
       <c r="AF11">
-        <v>0</v>
+        <v>1.02408650514922E-3</v>
       </c>
       <c r="AG11">
-        <v>0</v>
+        <v>1.98493598986983E-4</v>
       </c>
       <c r="AH11">
-        <v>0</v>
+        <v>2.0348430730881E-4</v>
       </c>
       <c r="AI11">
         <v>0</v>
@@ -79846,91 +79846,91 @@
         <v>11</v>
       </c>
       <c r="F12">
-        <v>1.2239147337734799E-70</v>
+        <v>1.1204846991804599E-10</v>
       </c>
       <c r="G12">
-        <v>9.5406589121923001E-63</v>
+        <v>9.7224750490505991E-10</v>
       </c>
       <c r="H12">
-        <v>2.4649930609334698E-55</v>
+        <v>7.4985444875915995E-9</v>
       </c>
       <c r="I12">
-        <v>2.11200269027871E-48</v>
+        <v>5.1406179026201798E-8</v>
       </c>
       <c r="J12">
-        <v>6.0047680141208506E-42</v>
+        <v>3.1325690783861401E-7</v>
       </c>
       <c r="K12">
-        <v>5.6698074019727499E-36</v>
+        <v>1.6968422431877999E-6</v>
       </c>
       <c r="L12">
-        <v>1.77969477385789E-30</v>
+        <v>8.1704494668440008E-6</v>
       </c>
       <c r="M12">
-        <v>1.85943735443383E-25</v>
+        <v>3.4972118631060003E-5</v>
       </c>
       <c r="N12">
-        <v>6.4773096292725003E-21</v>
+        <v>1.3306900405695899E-4</v>
       </c>
       <c r="O12">
-        <v>7.5393830513013606E-17</v>
+        <v>4.50109174154029E-4</v>
       </c>
       <c r="P12">
-        <v>2.9409708584991399E-13</v>
+        <v>1.35347854430027E-3</v>
       </c>
       <c r="Q12">
-        <v>3.8603951586587002E-10</v>
+        <v>3.61812435954963E-3</v>
       </c>
       <c r="R12">
-        <v>1.7148886469501001E-7</v>
+        <v>8.5984410349495503E-3</v>
       </c>
       <c r="S12">
-        <v>2.5987779114898801E-5</v>
+        <v>1.8166237654753899E-2</v>
       </c>
       <c r="T12">
-        <v>1.35824215419107E-3</v>
+        <v>3.41211484325682E-2</v>
       </c>
       <c r="U12">
-        <v>2.4830306488605201E-2</v>
+        <v>5.69769710006955E-2</v>
       </c>
       <c r="V12">
-        <v>0.161357600311022</v>
+        <v>8.4585356069357603E-2</v>
       </c>
       <c r="W12">
-        <v>0.37828433079052098</v>
+        <v>0.11163836656981301</v>
       </c>
       <c r="X12">
-        <v>0.32263549087555599</v>
+        <v>0.13099535654899</v>
       </c>
       <c r="Y12">
-        <v>9.9942284300248194E-2</v>
+        <v>0.136654340535355</v>
       </c>
       <c r="Z12">
-        <v>1.11218634639916E-2</v>
+        <v>0.12674076306597201</v>
       </c>
       <c r="AA12">
-        <v>4.3769712873609201E-4</v>
+        <v>0.104504286965027</v>
       </c>
       <c r="AB12">
-        <v>5.99656095412459E-6</v>
+        <v>7.6608266201317901E-2</v>
       </c>
       <c r="AC12">
-        <v>2.822663613955E-8</v>
+        <v>4.99274096589363E-2</v>
       </c>
       <c r="AD12">
-        <v>4.5198844667027002E-11</v>
+        <v>2.8928223012135601E-2</v>
       </c>
       <c r="AE12">
-        <v>2.44249065417534E-14</v>
+        <v>1.4901177101189E-2</v>
       </c>
       <c r="AF12">
-        <v>0</v>
+        <v>6.8238837258766403E-3</v>
       </c>
       <c r="AG12">
-        <v>0</v>
+        <v>1.71764721676139E-3</v>
       </c>
       <c r="AH12">
-        <v>0</v>
+        <v>2.5121314679717398E-3</v>
       </c>
       <c r="AI12">
         <v>0</v>
@@ -80214,91 +80214,91 @@
         <v>12</v>
       </c>
       <c r="F13">
-        <v>1.6473275959227299E-65</v>
+        <v>1.34905555737526E-10</v>
       </c>
       <c r="G13">
-        <v>1.52157216315028E-58</v>
+        <v>1.02623790026422E-9</v>
       </c>
       <c r="H13">
-        <v>5.5645771175117797E-52</v>
+        <v>7.0297676044139303E-9</v>
       </c>
       <c r="I13">
-        <v>8.0611145471316502E-46</v>
+        <v>4.3362543791540198E-8</v>
       </c>
       <c r="J13">
-        <v>4.6282584682337901E-40</v>
+        <v>2.4086594201646601E-7</v>
       </c>
       <c r="K13">
-        <v>1.0538707472209599E-34</v>
+        <v>1.20483814715222E-6</v>
       </c>
       <c r="L13">
-        <v>9.5248683002705694E-30</v>
+        <v>5.4272557763661802E-6</v>
       </c>
       <c r="M13">
-        <v>3.4203914932387901E-25</v>
+        <v>2.2015852121264001E-5</v>
       </c>
       <c r="N13">
-        <v>4.8865262920401898E-21</v>
+        <v>8.0426551282892903E-5</v>
       </c>
       <c r="O13">
-        <v>2.7819959315550902E-17</v>
+        <v>2.6459215228774097E-4</v>
       </c>
       <c r="P13">
-        <v>6.3254411391713404E-14</v>
+        <v>7.8392148189435204E-4</v>
       </c>
       <c r="Q13">
-        <v>5.7604224287047197E-11</v>
+        <v>2.0916570255723401E-3</v>
       </c>
       <c r="R13">
-        <v>2.10917188153067E-8</v>
+        <v>5.0261396323154801E-3</v>
       </c>
       <c r="S13">
-        <v>3.12084561546368E-6</v>
+        <v>1.08769792738677E-2</v>
       </c>
       <c r="T13">
-        <v>1.8784951960861099E-4</v>
+        <v>2.1198974792711399E-2</v>
       </c>
       <c r="U13">
-        <v>4.6377883084965498E-3</v>
+        <v>3.72097678787362E-2</v>
       </c>
       <c r="V13">
-        <v>4.7414453579626002E-2</v>
+        <v>5.8821614558663499E-2</v>
       </c>
       <c r="W13">
-        <v>0.202669863207316</v>
+        <v>8.3744581028296503E-2</v>
       </c>
       <c r="X13">
-        <v>0.36500474681893602</v>
+        <v>0.10737860749117099</v>
       </c>
       <c r="Y13">
-        <v>0.27797542378274898</v>
+        <v>0.12399984819739999</v>
       </c>
       <c r="Z13">
-        <v>8.9365583499576004E-2</v>
+        <v>0.12896369944007099</v>
       </c>
       <c r="AA13">
-        <v>1.2050151430856099E-2</v>
+        <v>0.12079721519754</v>
       </c>
       <c r="AB13">
-        <v>6.7527656580568197E-4</v>
+        <v>0.10190352195407799</v>
       </c>
       <c r="AC13">
-        <v>1.55741973125733E-5</v>
+        <v>7.7421855694793498E-2</v>
       </c>
       <c r="AD13">
-        <v>1.46535444445206E-7</v>
+        <v>5.2975968838959803E-2</v>
       </c>
       <c r="AE13">
-        <v>5.58411983320183E-10</v>
+        <v>3.2646271889236599E-2</v>
       </c>
       <c r="AF13">
-        <v>8.5698115270815803E-13</v>
+        <v>1.8118640660344399E-2</v>
       </c>
       <c r="AG13">
-        <v>5.5511151231257797E-16</v>
+        <v>5.3681626153421298E-3</v>
       </c>
       <c r="AH13">
-        <v>0</v>
+        <v>1.0298613279994E-2</v>
       </c>
       <c r="AI13">
         <v>0</v>
@@ -80582,91 +80582,91 @@
         <v>13</v>
       </c>
       <c r="F14">
-        <v>1.8571594341261001E-59</v>
+        <v>1.7873873436799099E-11</v>
       </c>
       <c r="G14">
-        <v>2.1411213937556702E-53</v>
+        <v>1.4286912193088E-10</v>
       </c>
       <c r="H14">
-        <v>1.1393736122818299E-47</v>
+        <v>1.0333411519358899E-9</v>
       </c>
       <c r="I14">
-        <v>2.7995916434507101E-42</v>
+        <v>6.76301158944471E-9</v>
       </c>
       <c r="J14">
-        <v>3.17783097647404E-37</v>
+        <v>4.0052799198518397E-8</v>
       </c>
       <c r="K14">
-        <v>1.6673235306153799E-32</v>
+        <v>2.1464811759446901E-7</v>
       </c>
       <c r="L14">
-        <v>4.0463210544934396E-28</v>
+        <v>1.0409448863255E-6</v>
       </c>
       <c r="M14">
-        <v>4.5458895736104797E-24</v>
+        <v>4.5681422630257498E-6</v>
       </c>
       <c r="N14">
-        <v>2.36674239498118E-20</v>
+        <v>1.8141255110712501E-5</v>
       </c>
       <c r="O14">
-        <v>5.7177882460114501E-17</v>
+        <v>6.5195143237825899E-5</v>
       </c>
       <c r="P14">
-        <v>6.4205595621567895E-14</v>
+        <v>2.12025210895329E-4</v>
       </c>
       <c r="Q14">
-        <v>3.35818241918685E-11</v>
+        <v>6.2400490587469898E-4</v>
       </c>
       <c r="R14">
-        <v>8.2033305618029701E-9</v>
+        <v>1.66195925080492E-3</v>
       </c>
       <c r="S14">
-        <v>9.3908107027799598E-7</v>
+        <v>4.0057878944069498E-3</v>
       </c>
       <c r="T14">
-        <v>5.0589789445272099E-5</v>
+        <v>8.7376327596603003E-3</v>
       </c>
       <c r="U14">
-        <v>1.28896006635537E-3</v>
+        <v>1.7248074593770198E-2</v>
       </c>
       <c r="V14">
-        <v>1.5619684950406099E-2</v>
+        <v>3.08127788705857E-2</v>
       </c>
       <c r="W14">
-        <v>9.0544863807600504E-2</v>
+        <v>4.9815742159396201E-2</v>
       </c>
       <c r="X14">
-        <v>0.25236906783482199</v>
+        <v>7.2886915578336403E-2</v>
       </c>
       <c r="Y14">
-        <v>0.33940057889401298</v>
+        <v>9.6511964362572297E-2</v>
       </c>
       <c r="Z14">
-        <v>0.22048045765552499</v>
+        <v>0.115654459052667</v>
       </c>
       <c r="AA14">
-        <v>6.9074865522275306E-2</v>
+        <v>0.12542783225679599</v>
       </c>
       <c r="AB14">
-        <v>1.0396295287165101E-2</v>
+        <v>0.123105103756439</v>
       </c>
       <c r="AC14">
-        <v>7.4772306352788298E-4</v>
+        <v>0.10934746991540401</v>
       </c>
       <c r="AD14">
-        <v>2.5550156467990499E-5</v>
+        <v>8.7900535562870197E-2</v>
       </c>
       <c r="AE14">
-        <v>4.12511636405099E-7</v>
+        <v>6.3947504976549899E-2</v>
       </c>
       <c r="AF14">
-        <v>3.1315603443715599E-9</v>
+        <v>4.21021065298064E-2</v>
       </c>
       <c r="AG14">
-        <v>1.0652034809766E-11</v>
+        <v>1.43222406615541E-2</v>
       </c>
       <c r="AH14">
-        <v>4.9948933877885702E-13</v>
+        <v>3.5586653558100201E-2</v>
       </c>
       <c r="AI14">
         <v>0</v>
@@ -80950,91 +80950,91 @@
         <v>14</v>
       </c>
       <c r="F15">
-        <v>4.7634196532531597E-46</v>
+        <v>6.8748694525000697E-10</v>
       </c>
       <c r="G15">
-        <v>1.5142495925781901E-41</v>
+        <v>3.7021706223558601E-9</v>
       </c>
       <c r="H15">
-        <v>2.7672919231777899E-37</v>
+        <v>1.8430773792140999E-8</v>
       </c>
       <c r="I15">
-        <v>2.90824986758116E-33</v>
+        <v>8.4825848517998194E-8</v>
       </c>
       <c r="J15">
-        <v>1.7583339241146101E-29</v>
+        <v>3.6092139680616801E-7</v>
       </c>
       <c r="K15">
-        <v>6.1188311215877003E-26</v>
+        <v>1.41970793352288E-6</v>
       </c>
       <c r="L15">
-        <v>1.2262390827816301E-22</v>
+        <v>5.1628494151491999E-6</v>
       </c>
       <c r="M15">
-        <v>1.41614904495765E-19</v>
+        <v>1.7357452831679899E-5</v>
       </c>
       <c r="N15">
-        <v>9.4321817145494799E-17</v>
+        <v>5.3949887040925198E-5</v>
       </c>
       <c r="O15">
-        <v>3.6265374507434102E-14</v>
+        <v>1.55026135484093E-4</v>
       </c>
       <c r="P15">
-        <v>8.0581004678438105E-12</v>
+        <v>4.1184221325957698E-4</v>
       </c>
       <c r="Q15">
-        <v>1.0361061728846E-9</v>
+        <v>1.0115095037027701E-3</v>
       </c>
       <c r="R15">
-        <v>7.7209809983710193E-8</v>
+        <v>2.2968030028945401E-3</v>
       </c>
       <c r="S15">
-        <v>3.3404148819460502E-6</v>
+        <v>4.8216266941136701E-3</v>
       </c>
       <c r="T15">
-        <v>8.4070029746405195E-5</v>
+        <v>9.3579503891495098E-3</v>
       </c>
       <c r="U15">
-        <v>1.23343381926311E-3</v>
+        <v>1.6791378619881E-2</v>
       </c>
       <c r="V15">
-        <v>1.0572354345068299E-2</v>
+        <v>2.7855531143372501E-2</v>
       </c>
       <c r="W15">
-        <v>5.30542605759294E-2</v>
+        <v>4.27225227932354E-2</v>
       </c>
       <c r="X15">
-        <v>0.15615582772900399</v>
+        <v>6.05791874440079E-2</v>
       </c>
       <c r="Y15">
-        <v>0.269949699818547</v>
+        <v>7.9416678762016399E-2</v>
       </c>
       <c r="Z15">
-        <v>0.27429590347057897</v>
+        <v>9.6254756649421694E-2</v>
       </c>
       <c r="AA15">
-        <v>0.16382392993089401</v>
+        <v>0.107858710585182</v>
       </c>
       <c r="AB15">
-        <v>5.7471155278057601E-2</v>
+        <v>0.111740598852357</v>
       </c>
       <c r="AC15">
-        <v>1.1826446215248299E-2</v>
+        <v>0.107026069051151</v>
       </c>
       <c r="AD15">
-        <v>1.4249620031825301E-3</v>
+        <v>9.4774365904271601E-2</v>
       </c>
       <c r="AE15">
-        <v>1.00320584685009E-4</v>
+        <v>7.7591601681910802E-2</v>
       </c>
       <c r="AF15">
-        <v>4.11782061482401E-6</v>
+        <v>5.8730095599177898E-2</v>
       </c>
       <c r="AG15">
-        <v>8.7183523622691399E-8</v>
+        <v>2.2588146479053502E-2</v>
       </c>
       <c r="AH15">
-        <v>1.25267632933301E-8</v>
+        <v>7.7937240031459104E-2</v>
       </c>
       <c r="AI15">
         <v>0</v>
@@ -81318,91 +81318,91 @@
         <v>15</v>
       </c>
       <c r="F16">
-        <v>2.1520332814873201E-43</v>
+        <v>1.70207758960061E-12</v>
       </c>
       <c r="G16">
-        <v>2.8303579125063699E-39</v>
+        <v>1.4812735577065401E-11</v>
       </c>
       <c r="H16">
-        <v>2.2761858911959999E-35</v>
+        <v>1.1688802680024599E-10</v>
       </c>
       <c r="I16">
-        <v>1.1195937290261201E-31</v>
+        <v>8.3635140182845497E-10</v>
       </c>
       <c r="J16">
-        <v>3.3694050432547499E-28</v>
+        <v>5.4262102622469997E-9</v>
       </c>
       <c r="K16">
-        <v>6.2067576956336296E-25</v>
+        <v>3.1922614967860698E-8</v>
       </c>
       <c r="L16">
-        <v>7.0017029200796896E-22</v>
+        <v>1.7029391272505499E-7</v>
       </c>
       <c r="M16">
-        <v>4.83964443503723E-19</v>
+        <v>8.2376487939673099E-7</v>
       </c>
       <c r="N16">
-        <v>2.0510612787253301E-16</v>
+        <v>3.61339466036741E-6</v>
       </c>
       <c r="O16">
-        <v>5.3337286410540898E-14</v>
+        <v>1.43727481185318E-5</v>
       </c>
       <c r="P16">
-        <v>8.5183456857576994E-12</v>
+        <v>5.1841867060549302E-5</v>
       </c>
       <c r="Q16">
-        <v>8.3636341120819405E-10</v>
+        <v>1.69567163577243E-4</v>
       </c>
       <c r="R16">
-        <v>5.0542288013716298E-8</v>
+        <v>5.0295235814411699E-4</v>
       </c>
       <c r="S16">
-        <v>1.88234795827243E-6</v>
+        <v>1.35281789246105E-3</v>
       </c>
       <c r="T16">
-        <v>4.3266164459440798E-5</v>
+        <v>3.2997602932632701E-3</v>
       </c>
       <c r="U16">
-        <v>6.14690829188588E-4</v>
+        <v>7.2989250671480297E-3</v>
       </c>
       <c r="V16">
-        <v>5.4062235397287399E-3</v>
+        <v>1.4641025218864101E-2</v>
       </c>
       <c r="W16">
-        <v>2.94785609365978E-2</v>
+        <v>2.6633145375117101E-2</v>
       </c>
       <c r="X16">
-        <v>9.9786662091955802E-2</v>
+        <v>4.3935323575670801E-2</v>
       </c>
       <c r="Y16">
-        <v>0.20992136958278301</v>
+        <v>6.5727527353815707E-2</v>
       </c>
       <c r="Z16">
-        <v>0.274640081873049</v>
+        <v>8.9171121954279994E-2</v>
       </c>
       <c r="AA16">
-        <v>0.22351621470313901</v>
+        <v>0.109709866293211</v>
       </c>
       <c r="AB16">
-        <v>0.11313678530414301</v>
+        <v>0.122408724746414</v>
       </c>
       <c r="AC16">
-        <v>3.5593186015515497E-2</v>
+        <v>0.12385817387332899</v>
       </c>
       <c r="AD16">
-        <v>6.9526886150418302E-3</v>
+        <v>0.11365345011441599</v>
       </c>
       <c r="AE16">
-        <v>8.4216096333344904E-4</v>
+        <v>9.4577086253767997E-2</v>
       </c>
       <c r="AF16">
-        <v>6.3161722466897804E-5</v>
+        <v>7.1373000916434906E-2</v>
       </c>
       <c r="AG16">
-        <v>2.4756239941359201E-6</v>
+        <v>2.7042868541408801E-2</v>
       </c>
       <c r="AH16">
-        <v>5.3829942103789097E-7</v>
+        <v>8.4573802621464897E-2</v>
       </c>
       <c r="AI16">
         <v>0</v>
@@ -81686,91 +81686,91 @@
         <v>16</v>
       </c>
       <c r="F17">
-        <v>7.1842071489909104E-37</v>
+        <v>6.5817859874041499E-13</v>
       </c>
       <c r="G17">
-        <v>1.7828149174642001E-33</v>
+        <v>5.90318524530018E-12</v>
       </c>
       <c r="H17">
-        <v>2.98090982539432E-30</v>
+        <v>4.8056320756967398E-11</v>
       </c>
       <c r="I17">
-        <v>3.3581606121251204E-27</v>
+        <v>3.55092178267549E-10</v>
       </c>
       <c r="J17">
-        <v>2.5497166729973299E-24</v>
+        <v>2.3815687106352899E-9</v>
       </c>
       <c r="K17">
-        <v>1.3051640588336001E-21</v>
+        <v>1.4498443423598301E-8</v>
       </c>
       <c r="L17">
-        <v>4.5059369678419098E-19</v>
+        <v>8.0116247784851898E-8</v>
       </c>
       <c r="M17">
-        <v>1.04963279879724E-16</v>
+        <v>4.0185127833371599E-7</v>
       </c>
       <c r="N17">
-        <v>1.65055779635333E-14</v>
+        <v>1.8296164375991501E-6</v>
       </c>
       <c r="O17">
-        <v>1.75306856223245E-12</v>
+        <v>7.5615172150610904E-6</v>
       </c>
       <c r="P17">
-        <v>1.2583504100721299E-10</v>
+        <v>2.8367175257852699E-5</v>
       </c>
       <c r="Q17">
-        <v>6.1083568031133701E-9</v>
+        <v>9.6601830476303902E-5</v>
       </c>
       <c r="R17">
-        <v>2.00667565194918E-7</v>
+        <v>2.98621027557825E-4</v>
       </c>
       <c r="S17">
-        <v>4.4646817846746903E-6</v>
+        <v>8.37962533554222E-4</v>
       </c>
       <c r="T17">
-        <v>6.7330143864200698E-5</v>
+        <v>2.1345246810594298E-3</v>
       </c>
       <c r="U17">
-        <v>6.8878723714555E-4</v>
+        <v>4.9357487912768802E-3</v>
       </c>
       <c r="V17">
-        <v>4.7836763040836902E-3</v>
+        <v>1.03605511365E-2</v>
       </c>
       <c r="W17">
-        <v>2.2571668696145599E-2</v>
+        <v>1.97420838199391E-2</v>
       </c>
       <c r="X17">
-        <v>7.2406596044466198E-2</v>
+        <v>3.4149593353722703E-2</v>
       </c>
       <c r="Y17">
-        <v>0.15799363495305099</v>
+        <v>5.3624380340539297E-2</v>
       </c>
       <c r="Z17">
-        <v>0.234592818903647</v>
+        <v>7.6440713074677605E-2</v>
       </c>
       <c r="AA17">
-        <v>0.237077926069937</v>
+        <v>9.8917707273530095E-2</v>
       </c>
       <c r="AB17">
-        <v>0.16306891206062901</v>
+        <v>0.11620132545586399</v>
       </c>
       <c r="AC17">
-        <v>7.6325879746236294E-2</v>
+        <v>0.123918568793949</v>
       </c>
       <c r="AD17">
-        <v>2.4301353635247901E-2</v>
+        <v>0.119963790034952</v>
       </c>
       <c r="AE17">
-        <v>5.26036707836174E-3</v>
+        <v>0.105427119478301</v>
       </c>
       <c r="AF17">
-        <v>7.7364846585414805E-4</v>
+        <v>8.4108995170146097E-2</v>
       </c>
       <c r="AG17">
-        <v>6.0401106371177301E-5</v>
+        <v>3.3291213155173603E-2</v>
       </c>
       <c r="AH17">
-        <v>2.2327969645852199E-5</v>
+        <v>0.115512242482623</v>
       </c>
       <c r="AI17">
         <v>0</v>
@@ -82054,91 +82054,91 @@
         <v>17</v>
       </c>
       <c r="F18">
-        <v>4.33744718482014E-63</v>
+        <v>2.93842708498843E-12</v>
       </c>
       <c r="G18">
-        <v>2.8903174401931899E-57</v>
+        <v>2.1845396578760699E-11</v>
       </c>
       <c r="H18">
-        <v>9.8759384390576106E-52</v>
+        <v>1.4901408824230699E-10</v>
       </c>
       <c r="I18">
-        <v>1.7308308172496699E-46</v>
+        <v>9.326538875956691E-10</v>
       </c>
       <c r="J18">
-        <v>1.5563856745732099E-41</v>
+        <v>5.3560272791254203E-9</v>
       </c>
       <c r="K18">
-        <v>7.1834749031267999E-37</v>
+        <v>2.8222624358648801E-8</v>
       </c>
       <c r="L18">
-        <v>1.70257637182323E-32</v>
+        <v>1.3645438546950399E-7</v>
       </c>
       <c r="M18">
-        <v>2.0733497735637499E-28</v>
+        <v>6.0536336593633504E-7</v>
       </c>
       <c r="N18">
-        <v>1.29813896915014E-24</v>
+        <v>2.4642584150719998E-6</v>
       </c>
       <c r="O18">
-        <v>4.18218670309463E-21</v>
+        <v>9.2045096668114608E-6</v>
       </c>
       <c r="P18">
-        <v>6.9398294593315002E-18</v>
+        <v>3.1547290350900801E-5</v>
       </c>
       <c r="Q18">
-        <v>5.9386209258058499E-15</v>
+        <v>9.92140154119254E-5</v>
       </c>
       <c r="R18">
-        <v>2.6246109933659099E-12</v>
+        <v>2.8630964159995101E-4</v>
       </c>
       <c r="S18">
-        <v>6.0018862648145902E-10</v>
+        <v>7.5814657445802695E-4</v>
       </c>
       <c r="T18">
-        <v>7.1175694592480399E-8</v>
+        <v>1.84215749284882E-3</v>
       </c>
       <c r="U18">
-        <v>4.3890604387364298E-6</v>
+        <v>4.1073212214214E-3</v>
       </c>
       <c r="V18">
-        <v>1.4118291287685099E-4</v>
+        <v>8.4033161061990696E-3</v>
       </c>
       <c r="W18">
-        <v>2.3774331472328799E-3</v>
+        <v>1.5776274840947901E-2</v>
       </c>
       <c r="X18">
-        <v>2.1037047988677199E-2</v>
+        <v>2.717824375021E-2</v>
       </c>
       <c r="Y18">
-        <v>9.8173753091246999E-2</v>
+        <v>4.29638037272628E-2</v>
       </c>
       <c r="Z18">
-        <v>0.242370967448229</v>
+        <v>6.2323168351325703E-2</v>
       </c>
       <c r="AA18">
-        <v>0.31719861886927703</v>
+        <v>8.2958836312579096E-2</v>
       </c>
       <c r="AB18">
-        <v>0.22020621860481299</v>
+        <v>0.101331103885485</v>
       </c>
       <c r="AC18">
-        <v>8.10204676238446E-2</v>
+        <v>0.113576990940418</v>
       </c>
       <c r="AD18">
-        <v>1.5763613308629899E-2</v>
+        <v>0.116816898853091</v>
       </c>
       <c r="AE18">
-        <v>1.61667175335022E-3</v>
+        <v>0.11025258549365299</v>
       </c>
       <c r="AF18">
-        <v>8.7074325675229298E-5</v>
+        <v>9.5485967451142295E-2</v>
       </c>
       <c r="AG18">
-        <v>2.1639308297460798E-6</v>
+        <v>4.0539706742701097E-2</v>
       </c>
       <c r="AH18">
-        <v>3.2615636302857301E-7</v>
+        <v>0.17525596203795801</v>
       </c>
       <c r="AI18">
         <v>0</v>
@@ -82422,91 +82422,91 @@
         <v>18</v>
       </c>
       <c r="F19">
-        <v>1.19520557740487E-33</v>
+        <v>4.0007120292543297E-11</v>
       </c>
       <c r="G19">
-        <v>1.1304344126301901E-30</v>
+        <v>2.19756301451678E-10</v>
       </c>
       <c r="H19">
-        <v>7.66608381986315E-28</v>
+        <v>1.1258620331739499E-9</v>
       </c>
       <c r="I19">
-        <v>3.7255413165533998E-25</v>
+        <v>5.3798535354117001E-9</v>
       </c>
       <c r="J19">
-        <v>1.29775834982839E-22</v>
+        <v>2.39772172795302E-8</v>
       </c>
       <c r="K19">
-        <v>3.2411483204990699E-20</v>
+        <v>9.96716650084147E-8</v>
       </c>
       <c r="L19">
-        <v>5.8053508186654997E-18</v>
+        <v>3.8644773433947398E-7</v>
       </c>
       <c r="M19">
-        <v>7.4596593747462098E-16</v>
+        <v>1.39751794533746E-6</v>
       </c>
       <c r="N19">
-        <v>6.8789175768319604E-14</v>
+        <v>4.7138200467081803E-6</v>
       </c>
       <c r="O19">
-        <v>4.5540182628260398E-12</v>
+        <v>1.4829924048274601E-5</v>
       </c>
       <c r="P19">
-        <v>2.1653049363959199E-10</v>
+        <v>4.35167506928047E-5</v>
       </c>
       <c r="Q19">
-        <v>7.39743809472674E-9</v>
+        <v>1.1910412932146301E-4</v>
       </c>
       <c r="R19">
-        <v>1.8166889086596801E-7</v>
+        <v>3.04054304937753E-4</v>
       </c>
       <c r="S19">
-        <v>3.2086608770163398E-6</v>
+        <v>7.2398665288555002E-4</v>
       </c>
       <c r="T19">
-        <v>4.0777698863569303E-5</v>
+        <v>1.6079259444211999E-3</v>
       </c>
       <c r="U19">
-        <v>3.73068647965437E-4</v>
+        <v>3.3308766306610299E-3</v>
       </c>
       <c r="V19">
-        <v>2.4582591032698501E-3</v>
+        <v>6.43589486802179E-3</v>
       </c>
       <c r="W19">
-        <v>1.1671665730135001E-2</v>
+        <v>1.1598932304309299E-2</v>
       </c>
       <c r="X19">
-        <v>3.9946467538668699E-2</v>
+        <v>1.94978388532022E-2</v>
       </c>
       <c r="Y19">
-        <v>9.85852402826735E-2</v>
+        <v>3.05713742209173E-2</v>
       </c>
       <c r="Z19">
-        <v>0.17548822417720999</v>
+        <v>4.4709932778934099E-2</v>
       </c>
       <c r="AA19">
-        <v>0.22535265576777</v>
+        <v>6.0989364810155301E-2</v>
       </c>
       <c r="AB19">
-        <v>0.20878040092591499</v>
+        <v>7.7600697351934103E-2</v>
       </c>
       <c r="AC19">
-        <v>0.13954644308936701</v>
+        <v>9.2095594515126097E-2</v>
       </c>
       <c r="AD19">
-        <v>6.7281540720425206E-2</v>
+        <v>0.10194689845822399</v>
       </c>
       <c r="AE19">
-        <v>2.3395187163099001E-2</v>
+        <v>0.10526190753289601</v>
       </c>
       <c r="AF19">
-        <v>5.8651584710866997E-3</v>
+        <v>0.101374925990126</v>
       </c>
       <c r="AG19">
-        <v>7.6546193759940897E-4</v>
+        <v>4.7156086450832697E-2</v>
       </c>
       <c r="AH19">
-        <v>4.4605079759008E-4</v>
+        <v>0.29460962932826501</v>
       </c>
       <c r="AI19">
         <v>0</v>
@@ -82790,91 +82790,91 @@
         <v>19</v>
       </c>
       <c r="F20">
-        <v>1.9371099832072099E-30</v>
+        <v>1.14575402387767E-13</v>
       </c>
       <c r="G20">
-        <v>8.4406508777080103E-28</v>
+        <v>1.0184943693929099E-12</v>
       </c>
       <c r="H20">
-        <v>2.7534819367336801E-25</v>
+        <v>8.2753588205579494E-12</v>
       </c>
       <c r="I20">
-        <v>6.7143797277667296E-23</v>
+        <v>6.1458224361650197E-11</v>
       </c>
       <c r="J20">
-        <v>1.2241384103550999E-20</v>
+        <v>4.1719788737079699E-10</v>
       </c>
       <c r="K20">
-        <v>1.6689644803311399E-18</v>
+        <v>2.5886716961644099E-9</v>
       </c>
       <c r="L20">
-        <v>1.7019792666229299E-16</v>
+        <v>1.4682107810596E-8</v>
       </c>
       <c r="M20">
-        <v>1.29854952709835E-14</v>
+        <v>7.6116722054613803E-8</v>
       </c>
       <c r="N20">
-        <v>7.4143674195526097E-13</v>
+        <v>3.6070781066180601E-7</v>
       </c>
       <c r="O20">
-        <v>3.1690037019129099E-11</v>
+        <v>1.562493651033E-6</v>
       </c>
       <c r="P20">
-        <v>1.01422203358242E-9</v>
+        <v>6.1868777545360401E-6</v>
       </c>
       <c r="Q20">
-        <v>2.4313051677760299E-8</v>
+        <v>2.2393322706956999E-5</v>
       </c>
       <c r="R20">
-        <v>4.36697809316305E-7</v>
+        <v>7.4090460096857196E-5</v>
       </c>
       <c r="S20">
-        <v>5.87894291757149E-6</v>
+        <v>2.24081318452035E-4</v>
       </c>
       <c r="T20">
-        <v>5.9338422464918998E-5</v>
+        <v>6.1951425262517397E-4</v>
       </c>
       <c r="U20">
-        <v>4.4919046387065697E-4</v>
+        <v>1.56567547783628E-3</v>
       </c>
       <c r="V20">
-        <v>2.5510342057330801E-3</v>
+        <v>3.6170899397219699E-3</v>
       </c>
       <c r="W20">
-        <v>1.08721981661192E-2</v>
+        <v>7.6388167816945898E-3</v>
       </c>
       <c r="X20">
-        <v>3.4781223337702998E-2</v>
+        <v>1.474701147285E-2</v>
       </c>
       <c r="Y20">
-        <v>8.3539765019775294E-2</v>
+        <v>2.6025242208577E-2</v>
       </c>
       <c r="Z20">
-        <v>0.150673590020764</v>
+        <v>4.1985551178880802E-2</v>
       </c>
       <c r="AA20">
-        <v>0.20409315906462999</v>
+        <v>6.19185118324787E-2</v>
       </c>
       <c r="AB20">
-        <v>0.20763208681831799</v>
+        <v>8.3475255839349602E-2</v>
       </c>
       <c r="AC20">
-        <v>0.158648787075058</v>
+        <v>0.10287560410519</v>
       </c>
       <c r="AD20">
-        <v>9.1039754601741102E-2</v>
+        <v>0.115900413543763</v>
       </c>
       <c r="AE20">
-        <v>3.9230909198320001E-2</v>
+        <v>0.119364680054869</v>
       </c>
       <c r="AF20">
-        <v>1.26927767483377E-2</v>
+        <v>0.112378966919409</v>
       </c>
       <c r="AG20">
-        <v>2.1223967290208098E-3</v>
+        <v>5.0727901126804198E-2</v>
       </c>
       <c r="AH20">
-        <v>1.60744912769617E-3</v>
+        <v>0.25683099620991201</v>
       </c>
       <c r="AI20">
         <v>0</v>
@@ -83158,91 +83158,91 @@
         <v>20</v>
       </c>
       <c r="F21">
-        <v>1.1967607320307E-43</v>
+        <v>5.8571488341412405E-14</v>
       </c>
       <c r="G21">
-        <v>7.7733679920467499E-40</v>
+        <v>5.1678181018571695E-13</v>
       </c>
       <c r="H21">
-        <v>3.32711721640159E-36</v>
+        <v>4.17922362684535E-12</v>
       </c>
       <c r="I21">
-        <v>9.3850867318089096E-33</v>
+        <v>3.0978121772139097E-11</v>
       </c>
       <c r="J21">
-        <v>1.7451459391164001E-29</v>
+        <v>2.10469525540356E-10</v>
       </c>
       <c r="K21">
-        <v>2.1398144657254401E-26</v>
+        <v>1.3106947083636E-9</v>
       </c>
       <c r="L21">
-        <v>1.73068116430747E-23</v>
+        <v>7.4816173699898998E-9</v>
       </c>
       <c r="M21">
-        <v>9.2367860955274795E-21</v>
+        <v>3.9144830366149701E-8</v>
       </c>
       <c r="N21">
-        <v>3.2544471990349601E-18</v>
+        <v>1.8773340904975599E-7</v>
       </c>
       <c r="O21">
-        <v>7.5735916855139795E-16</v>
+        <v>8.2527767326090295E-7</v>
       </c>
       <c r="P21">
-        <v>1.1647678900500399E-13</v>
+        <v>3.32547003000834E-6</v>
       </c>
       <c r="Q21">
-        <v>1.18458200223903E-11</v>
+        <v>1.22829675366583E-5</v>
       </c>
       <c r="R21">
-        <v>7.97235389237475E-10</v>
+        <v>4.15866246061049E-5</v>
       </c>
       <c r="S21">
-        <v>3.55339064766982E-8</v>
+        <v>1.2906449317672301E-4</v>
       </c>
       <c r="T21">
-        <v>1.0497910928892501E-6</v>
+        <v>3.67168248070244E-4</v>
       </c>
       <c r="U21">
-        <v>2.0575905595775498E-5</v>
+        <v>9.5748287383554999E-4</v>
       </c>
       <c r="V21">
-        <v>2.6780513524660003E-4</v>
+        <v>2.2887936463031801E-3</v>
       </c>
       <c r="W21">
-        <v>2.3168221303478801E-3</v>
+        <v>5.0152661590781604E-3</v>
       </c>
       <c r="X21">
-        <v>1.33344728464414E-2</v>
+        <v>1.00738358740457E-2</v>
       </c>
       <c r="Y21">
-        <v>5.1101023495307499E-2</v>
+        <v>1.85485910262536E-2</v>
       </c>
       <c r="Z21">
-        <v>0.13048469102751101</v>
+        <v>3.1307154096180803E-2</v>
       </c>
       <c r="AA21">
-        <v>0.22212392592824301</v>
+        <v>4.8438882109249098E-2</v>
       </c>
       <c r="AB21">
-        <v>0.25215855423888001</v>
+        <v>6.8701075122436103E-2</v>
       </c>
       <c r="AC21">
-        <v>0.190909696528647</v>
+        <v>8.9320819200040202E-2</v>
       </c>
       <c r="AD21">
-        <v>9.6379667820433196E-2</v>
+        <v>0.106454062217313</v>
       </c>
       <c r="AE21">
-        <v>3.2431939731803403E-2</v>
+        <v>0.116303445790336</v>
       </c>
       <c r="AF21">
-        <v>7.26993020965549E-3</v>
+        <v>0.11647801024971299</v>
       </c>
       <c r="AG21">
-        <v>8.0949124569529296E-4</v>
+        <v>5.5200032153865201E-2</v>
       </c>
       <c r="AH21">
-        <v>3.90317621991709E-4</v>
+        <v>0.33035806048350402</v>
       </c>
       <c r="AI21">
         <v>0</v>
@@ -83526,91 +83526,91 @@
         <v>21</v>
       </c>
       <c r="F22">
-        <v>2.39826284152207E-8</v>
+        <v>7.4227314481002198E-15</v>
       </c>
       <c r="G22">
-        <v>7.2930067652538999E-8</v>
+        <v>6.8775213939233705E-14</v>
       </c>
       <c r="H22">
-        <v>2.7104994859097701E-7</v>
+        <v>5.8544958337204104E-13</v>
       </c>
       <c r="I22">
-        <v>9.4496250567318197E-7</v>
+        <v>4.5786747019337498E-12</v>
       </c>
       <c r="J22">
-        <v>3.0903197704761001E-6</v>
+        <v>3.2899261758319601E-11</v>
       </c>
       <c r="K22">
-        <v>9.4801864412378406E-6</v>
+        <v>2.1718602210207E-10</v>
       </c>
       <c r="L22">
-        <v>2.7280726152673198E-5</v>
+        <v>1.31728625318068E-9</v>
       </c>
       <c r="M22">
-        <v>7.3641307800411497E-5</v>
+        <v>7.3406439744150903E-9</v>
       </c>
       <c r="N22">
-        <v>1.86472356785296E-4</v>
+        <v>3.7583475331189302E-8</v>
       </c>
       <c r="O22">
-        <v>4.4293057584436402E-4</v>
+        <v>1.7679560294158001E-7</v>
       </c>
       <c r="P22">
-        <v>9.8692892829329291E-4</v>
+        <v>7.6411830916194597E-7</v>
       </c>
       <c r="Q22">
-        <v>2.0628414277080701E-3</v>
+        <v>3.0343603036645302E-6</v>
       </c>
       <c r="R22">
-        <v>4.0446061338630804E-3</v>
+        <v>1.1071175774365599E-5</v>
       </c>
       <c r="S22">
-        <v>7.4390534116528699E-3</v>
+        <v>3.71144423685592E-5</v>
       </c>
       <c r="T22">
-        <v>1.28348481531522E-2</v>
+        <v>1.14318664631034E-4</v>
       </c>
       <c r="U22">
-        <v>2.0772842187287099E-2</v>
+        <v>3.23533036451041E-4</v>
       </c>
       <c r="V22">
-        <v>3.1537966756856897E-2</v>
+        <v>8.4129740696386502E-4</v>
       </c>
       <c r="W22">
-        <v>4.4916348029008901E-2</v>
+        <v>2.01007324207401E-3</v>
       </c>
       <c r="X22">
-        <v>6.0007909774711397E-2</v>
+        <v>4.4127311180764397E-3</v>
       </c>
       <c r="Y22">
-        <v>7.5204902226363293E-2</v>
+        <v>8.9009830673360598E-3</v>
       </c>
       <c r="Z22">
-        <v>8.8413301594683705E-2</v>
+        <v>1.6496997979586699E-2</v>
       </c>
       <c r="AA22">
-        <v>9.7504133560996298E-2</v>
+        <v>2.8093745518319099E-2</v>
       </c>
       <c r="AB22">
-        <v>0.100870111603027</v>
+        <v>4.3959557140615099E-2</v>
       </c>
       <c r="AC22">
-        <v>9.7889489329524501E-2</v>
+        <v>6.3202884706203499E-2</v>
       </c>
       <c r="AD22">
-        <v>8.9113537354248706E-2</v>
+        <v>8.3495145330198903E-2</v>
       </c>
       <c r="AE22">
-        <v>7.61001078820394E-2</v>
+        <v>0.10135073451495499</v>
       </c>
       <c r="AF22">
-        <v>6.0962206689854297E-2</v>
+        <v>0.11304057548726899</v>
       </c>
       <c r="AG22">
-        <v>2.4728201068473201E-2</v>
+        <v>5.8182476675713503E-2</v>
       </c>
       <c r="AH22">
-        <v>0.10386645549031</v>
+        <v>0.47552273872251699</v>
       </c>
       <c r="AI22">
         <v>0</v>
@@ -83894,25 +83894,25 @@
         <v>1</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>0.95114905762362001</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>4.7737387001594099E-2</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>1.1018710102991399E-3</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>1.1628411511944899E-5</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>5.5831390008575299E-8</v>
       </c>
       <c r="K23">
-        <v>0</v>
+        <v>1.2145453949637699E-10</v>
       </c>
       <c r="L23">
-        <v>0</v>
+        <v>1.2981459971823101E-13</v>
       </c>
       <c r="M23">
         <v>0</v>
@@ -84262,43 +84262,43 @@
         <v>2</v>
       </c>
       <c r="F24">
-        <v>0.82546043166524496</v>
+        <v>0.46577580638174998</v>
       </c>
       <c r="G24">
-        <v>0.172836716457412</v>
+        <v>0.334871926872922</v>
       </c>
       <c r="H24">
-        <v>1.70242065816594E-3</v>
+        <v>0.14973985160759001</v>
       </c>
       <c r="I24">
-        <v>4.3121679993429698E-7</v>
+        <v>4.1612660869892799E-2</v>
       </c>
       <c r="J24">
-        <v>2.37532216118552E-12</v>
+        <v>7.1789691605166697E-3</v>
       </c>
       <c r="K24">
-        <v>0</v>
+        <v>7.6781673965042798E-4</v>
       </c>
       <c r="L24">
-        <v>0</v>
+        <v>5.0834812084477099E-5</v>
       </c>
       <c r="M24">
-        <v>0</v>
+        <v>2.0801967698520902E-6</v>
       </c>
       <c r="N24">
-        <v>0</v>
+        <v>5.2533345232090997E-8</v>
       </c>
       <c r="O24">
-        <v>0</v>
+        <v>8.1760102113541504E-10</v>
       </c>
       <c r="P24">
-        <v>0</v>
+        <v>7.83187070891642E-12</v>
       </c>
       <c r="Q24">
-        <v>0</v>
+        <v>4.6129010404699601E-14</v>
       </c>
       <c r="R24">
-        <v>0</v>
+        <v>1.89831318537858E-16</v>
       </c>
       <c r="S24">
         <v>0</v>
@@ -84630,61 +84630,61 @@
         <v>3</v>
       </c>
       <c r="F25">
-        <v>1.59157363020795E-7</v>
+        <v>6.9277453233255903E-2</v>
       </c>
       <c r="G25">
-        <v>6.9066979169180303E-4</v>
+        <v>0.137715898491579</v>
       </c>
       <c r="H25">
-        <v>9.8767559684246498E-2</v>
+        <v>0.20353284051024201</v>
       </c>
       <c r="I25">
-        <v>0.63592206974564702</v>
+        <v>0.223656747540529</v>
       </c>
       <c r="J25">
-        <v>0.259123962495525</v>
+        <v>0.18274104405059999</v>
       </c>
       <c r="K25">
-        <v>5.4914193553577901E-3</v>
+        <v>0.111013681642219</v>
       </c>
       <c r="L25">
-        <v>4.1596760247397601E-6</v>
+        <v>5.0136502398389397E-2</v>
       </c>
       <c r="M25">
-        <v>9.4142804663022097E-11</v>
+        <v>1.6830330506359799E-2</v>
       </c>
       <c r="N25">
-        <v>1.11022302462515E-16</v>
+        <v>4.1984838742089399E-3</v>
       </c>
       <c r="O25">
-        <v>0</v>
+        <v>7.78096929439948E-4</v>
       </c>
       <c r="P25">
-        <v>0</v>
+        <v>1.07097819185152E-4</v>
       </c>
       <c r="Q25">
-        <v>0</v>
+        <v>1.09442548960273E-5</v>
       </c>
       <c r="R25">
-        <v>0</v>
+        <v>8.3003456237432398E-7</v>
       </c>
       <c r="S25">
-        <v>0</v>
+        <v>4.67038888360729E-8</v>
       </c>
       <c r="T25">
-        <v>0</v>
+        <v>1.9489443323656101E-9</v>
       </c>
       <c r="U25">
-        <v>0</v>
+        <v>6.0294883502423197E-11</v>
       </c>
       <c r="V25">
-        <v>0</v>
+        <v>1.3824853909768601E-12</v>
       </c>
       <c r="W25">
-        <v>0</v>
+        <v>2.3437797702923599E-14</v>
       </c>
       <c r="X25">
-        <v>0</v>
+        <v>3.4467349563122998E-16</v>
       </c>
       <c r="Y25">
         <v>0</v>
@@ -84998,73 +84998,73 @@
         <v>4</v>
       </c>
       <c r="F26">
-        <v>3.3339513310924801E-17</v>
+        <v>5.0173338467405099E-3</v>
       </c>
       <c r="G26">
-        <v>8.6932340519979599E-12</v>
+        <v>1.7008858475784198E-2</v>
       </c>
       <c r="H26">
-        <v>1.69723168137067E-7</v>
+        <v>4.5097322981773803E-2</v>
       </c>
       <c r="I26">
-        <v>2.5642831223617897E-4</v>
+        <v>9.3529993113765503E-2</v>
       </c>
       <c r="J26">
-        <v>3.2085166087999301E-2</v>
+        <v>0.15174525877644801</v>
       </c>
       <c r="K26">
-        <v>0.38016328335448502</v>
+        <v>0.19260622490697299</v>
       </c>
       <c r="L26">
-        <v>0.50751814695733799</v>
+        <v>0.19126253206758201</v>
       </c>
       <c r="M26">
-        <v>7.8760341517952595E-2</v>
+        <v>0.14859133339662201</v>
       </c>
       <c r="N26">
-        <v>1.2148667371945001E-3</v>
+        <v>9.0312287387384602E-2</v>
       </c>
       <c r="O26">
-        <v>1.5971361883027E-6</v>
+        <v>4.2940032472129297E-2</v>
       </c>
       <c r="P26">
-        <v>1.64742441910448E-10</v>
+        <v>1.5969812724348002E-2</v>
       </c>
       <c r="Q26">
-        <v>1.33226762955018E-15</v>
+        <v>4.6452326159561698E-3</v>
       </c>
       <c r="R26">
-        <v>0</v>
+        <v>1.05663119930173E-3</v>
       </c>
       <c r="S26">
-        <v>0</v>
+        <v>1.8792184682924699E-4</v>
       </c>
       <c r="T26">
-        <v>0</v>
+        <v>2.6127125898443501E-5</v>
       </c>
       <c r="U26">
-        <v>0</v>
+        <v>2.8391212784115601E-6</v>
       </c>
       <c r="V26">
-        <v>0</v>
+        <v>2.41083793821787E-7</v>
       </c>
       <c r="W26">
-        <v>0</v>
+        <v>1.5993946049735899E-8</v>
       </c>
       <c r="X26">
-        <v>0</v>
+        <v>8.2881549831964499E-10</v>
       </c>
       <c r="Y26">
-        <v>0</v>
+        <v>3.3541848393057598E-11</v>
       </c>
       <c r="Z26">
-        <v>0</v>
+        <v>1.0598564141752601E-12</v>
       </c>
       <c r="AA26">
-        <v>0</v>
+        <v>2.6126744711128199E-14</v>
       </c>
       <c r="AB26">
-        <v>0</v>
+        <v>5.5588818534315299E-16</v>
       </c>
       <c r="AC26">
         <v>0</v>
@@ -85366,79 +85366,79 @@
         <v>5</v>
       </c>
       <c r="F27">
-        <v>6.03040122745719E-38</v>
+        <v>9.6285897887483295E-5</v>
       </c>
       <c r="G27">
-        <v>1.71126723501641E-28</v>
+        <v>6.2477640112552403E-4</v>
       </c>
       <c r="H27">
-        <v>1.85678413646213E-20</v>
+        <v>3.1205213766410298E-3</v>
       </c>
       <c r="I27">
-        <v>7.7869898636986797E-14</v>
+        <v>1.19994063979057E-2</v>
       </c>
       <c r="J27">
-        <v>1.28635643397264E-8</v>
+        <v>3.5530548566064302E-2</v>
       </c>
       <c r="K27">
-        <v>8.6869467726121503E-5</v>
+        <v>8.1025358483885701E-2</v>
       </c>
       <c r="L27">
-        <v>2.60724134821585E-2</v>
+        <v>0.14232137354175001</v>
       </c>
       <c r="M27">
-        <v>0.42346257936159898</v>
+        <v>0.19256921191897</v>
       </c>
       <c r="N27">
-        <v>0.50460235478596205</v>
+        <v>0.20072044539803</v>
       </c>
       <c r="O27">
-        <v>4.5544147538489503E-2</v>
+        <v>0.161171122508311</v>
       </c>
       <c r="P27">
-        <v>2.3156918406197399E-4</v>
+        <v>9.9691653527713794E-2</v>
       </c>
       <c r="Q27">
-        <v>5.3315854176005901E-8</v>
+        <v>4.7497873005253398E-2</v>
       </c>
       <c r="R27">
-        <v>5.0581761001922102E-13</v>
+        <v>1.7429500996874899E-2</v>
       </c>
       <c r="S27">
-        <v>0</v>
+        <v>4.9252481340712802E-3</v>
       </c>
       <c r="T27">
-        <v>0</v>
+        <v>1.0715878529576001E-3</v>
       </c>
       <c r="U27">
-        <v>0</v>
+        <v>1.794722991301E-4</v>
       </c>
       <c r="V27">
-        <v>0</v>
+        <v>2.3133541913209301E-5</v>
       </c>
       <c r="W27">
-        <v>0</v>
+        <v>2.2943563822778801E-6</v>
       </c>
       <c r="X27">
-        <v>0</v>
+        <v>1.7504460847478399E-7</v>
       </c>
       <c r="Y27">
-        <v>0</v>
+        <v>1.02706730829322E-8</v>
       </c>
       <c r="Z27">
-        <v>0</v>
+        <v>4.6334506551212401E-10</v>
       </c>
       <c r="AA27">
-        <v>0</v>
+        <v>1.60679041915916E-11</v>
       </c>
       <c r="AB27">
-        <v>0</v>
+        <v>4.2821838982185998E-13</v>
       </c>
       <c r="AC27">
-        <v>0</v>
+        <v>8.7708718682724697E-15</v>
       </c>
       <c r="AD27">
-        <v>0</v>
+        <v>1.1102369453509501E-16</v>
       </c>
       <c r="AE27">
         <v>0</v>
@@ -85734,79 +85734,79 @@
         <v>6</v>
       </c>
       <c r="F28">
-        <v>7.5818358279871603E-40</v>
+        <v>1.09533126752395E-7</v>
       </c>
       <c r="G28">
-        <v>1.51397394243769E-31</v>
+        <v>2.0505249611784498E-6</v>
       </c>
       <c r="H28">
-        <v>2.9373080080001701E-24</v>
+        <v>2.7594641684386999E-5</v>
       </c>
       <c r="I28">
-        <v>5.5659825410091001E-18</v>
+        <v>2.67078044109103E-4</v>
       </c>
       <c r="J28">
-        <v>1.03847772893234E-12</v>
+        <v>1.86000522858224E-3</v>
       </c>
       <c r="K28">
-        <v>1.93317172512881E-8</v>
+        <v>9.3250302574886708E-3</v>
       </c>
       <c r="L28">
-        <v>3.6760954620576598E-5</v>
+        <v>3.36686463623731E-2</v>
       </c>
       <c r="M28">
-        <v>7.4692059361623798E-3</v>
+        <v>8.7577800283500304E-2</v>
       </c>
       <c r="N28">
-        <v>0.17663007079424001</v>
+        <v>0.164163519102596</v>
       </c>
       <c r="O28">
-        <v>0.55238634275661602</v>
+        <v>0.22179749724408401</v>
       </c>
       <c r="P28">
-        <v>0.24828514322847201</v>
+        <v>0.216010471621043</v>
       </c>
       <c r="Q28">
-        <v>1.5083552489779601E-2</v>
+        <v>0.151644803525009</v>
       </c>
       <c r="R28">
-        <v>1.08819654647818E-4</v>
+        <v>7.6730314712859904E-2</v>
       </c>
       <c r="S28">
-        <v>8.4845907077912801E-8</v>
+        <v>2.79771536906505E-2</v>
       </c>
       <c r="T28">
-        <v>6.7973404682675201E-12</v>
+        <v>7.3486954777665396E-3</v>
       </c>
       <c r="U28">
-        <v>0</v>
+        <v>1.3900450929670901E-3</v>
       </c>
       <c r="V28">
-        <v>0</v>
+        <v>1.8926781683239601E-4</v>
       </c>
       <c r="W28">
-        <v>0</v>
+        <v>1.8541892441530101E-5</v>
       </c>
       <c r="X28">
-        <v>0</v>
+        <v>1.30632347626394E-6</v>
       </c>
       <c r="Y28">
-        <v>0</v>
+        <v>6.6153521391427895E-8</v>
       </c>
       <c r="Z28">
-        <v>0</v>
+        <v>2.4068472874393102E-9</v>
       </c>
       <c r="AA28">
-        <v>0</v>
+        <v>6.2882699319647205E-11</v>
       </c>
       <c r="AB28">
-        <v>0</v>
+        <v>1.1792789018538101E-12</v>
       </c>
       <c r="AC28">
-        <v>0</v>
+        <v>1.5876189320758299E-14</v>
       </c>
       <c r="AD28">
-        <v>0</v>
+        <v>1.1102230294236601E-16</v>
       </c>
       <c r="AE28">
         <v>0</v>
@@ -86102,82 +86102,82 @@
         <v>7</v>
       </c>
       <c r="F29">
-        <v>9.8862227262646602E-104</v>
+        <v>1.4840805777608701E-9</v>
       </c>
       <c r="G29">
-        <v>4.9780584927305896E-84</v>
+        <v>4.4240972105360201E-8</v>
       </c>
       <c r="H29">
-        <v>1.93242031760028E-66</v>
+        <v>9.4062435325956401E-7</v>
       </c>
       <c r="I29">
-        <v>5.8031660570793596E-51</v>
+        <v>1.42711039891321E-5</v>
       </c>
       <c r="J29">
-        <v>1.35507213328866E-37</v>
+        <v>1.5458842965291301E-4</v>
       </c>
       <c r="K29">
-        <v>2.47980933663949E-26</v>
+        <v>1.19618896295585E-3</v>
       </c>
       <c r="L29">
-        <v>3.6035841309884699E-17</v>
+        <v>6.6151770543227198E-3</v>
       </c>
       <c r="M29">
-        <v>4.2600488430374602E-10</v>
+        <v>2.6157724262691098E-2</v>
       </c>
       <c r="N29">
-        <v>4.3138172913374902E-5</v>
+        <v>7.3985660531768499E-2</v>
       </c>
       <c r="O29">
-        <v>4.2891999014071099E-2</v>
+        <v>0.149734949373582</v>
       </c>
       <c r="P29">
-        <v>0.64537517253321097</v>
+        <v>0.21688302244593899</v>
       </c>
       <c r="Q29">
-        <v>0.30821989512033499</v>
+        <v>0.22485788088705499</v>
       </c>
       <c r="R29">
-        <v>3.46933560318596E-3</v>
+        <v>0.16686917381755301</v>
       </c>
       <c r="S29">
-        <v>4.5912972579387201E-7</v>
+        <v>8.8631149470195403E-2</v>
       </c>
       <c r="T29">
-        <v>5.5133675402885203E-13</v>
+        <v>3.3686012651709202E-2</v>
       </c>
       <c r="U29">
-        <v>0</v>
+        <v>9.1587252803192604E-3</v>
       </c>
       <c r="V29">
-        <v>0</v>
+        <v>1.7806432779802199E-3</v>
       </c>
       <c r="W29">
-        <v>0</v>
+        <v>2.47447008082376E-4</v>
       </c>
       <c r="X29">
-        <v>0</v>
+        <v>2.45662299899183E-5</v>
       </c>
       <c r="Y29">
-        <v>0</v>
+        <v>1.74149416482708E-6</v>
       </c>
       <c r="Z29">
-        <v>0</v>
+        <v>8.8105815091293805E-8</v>
       </c>
       <c r="AA29">
-        <v>0</v>
+        <v>3.1795063250055098E-9</v>
       </c>
       <c r="AB29">
-        <v>0</v>
+        <v>8.1802675747266698E-11</v>
       </c>
       <c r="AC29">
-        <v>0</v>
+        <v>1.49980028402027E-12</v>
       </c>
       <c r="AD29">
-        <v>0</v>
+        <v>1.9539925234108199E-14</v>
       </c>
       <c r="AE29">
-        <v>0</v>
+        <v>2.2204460493304702E-16</v>
       </c>
       <c r="AF29">
         <v>0</v>
@@ -86470,85 +86470,85 @@
         <v>8</v>
       </c>
       <c r="F30">
-        <v>9.8795791864220094E-145</v>
+        <v>4.2092772621216399E-11</v>
       </c>
       <c r="G30">
-        <v>2.2265533382672301E-119</v>
+        <v>1.6272336810069799E-9</v>
       </c>
       <c r="H30">
-        <v>1.6847938207329E-96</v>
+        <v>4.5377948435246498E-8</v>
       </c>
       <c r="I30">
-        <v>4.2912378012007203E-76</v>
+        <v>9.1325043009772598E-7</v>
       </c>
       <c r="J30">
-        <v>3.6922817557934499E-58</v>
+        <v>1.3270532549919301E-5</v>
       </c>
       <c r="K30">
-        <v>1.07887647209795E-42</v>
+        <v>1.3929816571179199E-4</v>
       </c>
       <c r="L30">
-        <v>1.079390331161E-29</v>
+        <v>1.0567274376336801E-3</v>
       </c>
       <c r="M30">
-        <v>3.7489373890866001E-19</v>
+        <v>5.7960754353755901E-3</v>
       </c>
       <c r="N30">
-        <v>4.6383505762978401E-11</v>
+        <v>2.2995132476746099E-2</v>
       </c>
       <c r="O30">
-        <v>2.1630131593569799E-5</v>
+        <v>6.6012128665355801E-2</v>
       </c>
       <c r="P30">
-        <v>4.4507427284404301E-2</v>
+        <v>0.13715883099909901</v>
       </c>
       <c r="Q30">
-        <v>0.70992239129337897</v>
+        <v>0.20631355291279799</v>
       </c>
       <c r="R30">
-        <v>0.24450488678530299</v>
+        <v>0.22469243668679201</v>
       </c>
       <c r="S30">
-        <v>1.0436415045272901E-3</v>
+        <v>0.17718095468768699</v>
       </c>
       <c r="T30">
-        <v>2.2954406264652502E-8</v>
+        <v>0.101153875145264</v>
       </c>
       <c r="U30">
-        <v>1.9984014443252802E-15</v>
+        <v>4.18035665542019E-2</v>
       </c>
       <c r="V30">
-        <v>0</v>
+        <v>1.25026136082548E-2</v>
       </c>
       <c r="W30">
-        <v>0</v>
+        <v>2.7052306879840498E-3</v>
       </c>
       <c r="X30">
-        <v>0</v>
+        <v>4.2330888409603402E-4</v>
       </c>
       <c r="Y30">
-        <v>0</v>
+        <v>4.78822445485853E-5</v>
       </c>
       <c r="Z30">
-        <v>0</v>
+        <v>3.9134311540265399E-6</v>
       </c>
       <c r="AA30">
-        <v>0</v>
+        <v>2.30995136130303E-7</v>
       </c>
       <c r="AB30">
-        <v>0</v>
+        <v>9.8424917105511297E-9</v>
       </c>
       <c r="AC30">
-        <v>0</v>
+        <v>3.0259605932083301E-10</v>
       </c>
       <c r="AD30">
-        <v>0</v>
+        <v>6.7094108047225497E-12</v>
       </c>
       <c r="AE30">
-        <v>0</v>
+        <v>1.07247544178875E-13</v>
       </c>
       <c r="AF30">
-        <v>0</v>
+        <v>1.2212453270886399E-15</v>
       </c>
       <c r="AG30">
         <v>0</v>
@@ -86838,91 +86838,91 @@
         <v>9</v>
       </c>
       <c r="F31">
-        <v>2.44148521576623E-89</v>
+        <v>5.5004216619428901E-12</v>
       </c>
       <c r="G31">
-        <v>8.9457634731663996E-75</v>
+        <v>2.3916195889876098E-10</v>
       </c>
       <c r="H31">
-        <v>1.5575063053845401E-61</v>
+        <v>7.5691677842634203E-9</v>
       </c>
       <c r="I31">
-        <v>1.2910799438016799E-49</v>
+        <v>1.7443858431684701E-7</v>
       </c>
       <c r="J31">
-        <v>5.1093421917559998E-39</v>
+        <v>2.9286008030574499E-6</v>
       </c>
       <c r="K31">
-        <v>9.6901957794990896E-30</v>
+        <v>3.5833485445376098E-5</v>
       </c>
       <c r="L31">
-        <v>8.8577376748747897E-22</v>
+        <v>3.1968077858957798E-4</v>
       </c>
       <c r="M31">
-        <v>3.9373014745905197E-15</v>
+        <v>2.0802928870306899E-3</v>
       </c>
       <c r="N31">
-        <v>8.6392186052802295E-10</v>
+        <v>9.8783403350933708E-3</v>
       </c>
       <c r="O31">
-        <v>9.6222073295791103E-6</v>
+        <v>3.4241237362202998E-2</v>
       </c>
       <c r="P31">
-        <v>5.7686801775611299E-3</v>
+        <v>8.6666818141518207E-2</v>
       </c>
       <c r="Q31">
-        <v>0.21270019670924101</v>
+        <v>0.16021319333261799</v>
       </c>
       <c r="R31">
-        <v>0.61567707597508503</v>
+        <v>0.21635022013251801</v>
       </c>
       <c r="S31">
-        <v>0.16256824113948201</v>
+        <v>0.213435123871687</v>
       </c>
       <c r="T31">
-        <v>3.2722137052421099E-3</v>
+        <v>0.15382335989766799</v>
       </c>
       <c r="U31">
-        <v>3.9689653397179097E-6</v>
+        <v>8.0981817982950302E-2</v>
       </c>
       <c r="V31">
-        <v>2.5679058879291001E-10</v>
+        <v>3.11377338473427E-2</v>
       </c>
       <c r="W31">
-        <v>8.8817841970012504E-16</v>
+        <v>8.7420652040085898E-3</v>
       </c>
       <c r="X31">
-        <v>0</v>
+        <v>1.7915729836507899E-3</v>
       </c>
       <c r="Y31">
-        <v>0</v>
+        <v>2.6791208169354698E-4</v>
       </c>
       <c r="Z31">
-        <v>0</v>
+        <v>2.92223548250564E-5</v>
       </c>
       <c r="AA31">
-        <v>0</v>
+        <v>2.3239172948221701E-6</v>
       </c>
       <c r="AB31">
-        <v>0</v>
+        <v>1.3468557769070899E-7</v>
       </c>
       <c r="AC31">
-        <v>0</v>
+        <v>5.68628433228522E-9</v>
       </c>
       <c r="AD31">
-        <v>0</v>
+        <v>1.74806946695599E-10</v>
       </c>
       <c r="AE31">
-        <v>0</v>
+        <v>3.9114267380572501E-12</v>
       </c>
       <c r="AF31">
-        <v>0</v>
+        <v>6.3615779311027402E-14</v>
       </c>
       <c r="AG31">
-        <v>0</v>
+        <v>6.6613381477515605E-16</v>
       </c>
       <c r="AH31">
-        <v>0</v>
+        <v>1.1102230246252601E-16</v>
       </c>
       <c r="AI31">
         <v>0</v>
@@ -87206,91 +87206,91 @@
         <v>10</v>
       </c>
       <c r="F32">
-        <v>1.1208596307891199E-96</v>
+        <v>2.06657661199966E-13</v>
       </c>
       <c r="G32">
-        <v>1.30112719574937E-81</v>
+        <v>1.2328479370863899E-11</v>
       </c>
       <c r="H32">
-        <v>7.5534504589156103E-68</v>
+        <v>5.3000455892570898E-10</v>
       </c>
       <c r="I32">
-        <v>2.1966337285801199E-55</v>
+        <v>1.6426611571409499E-8</v>
       </c>
       <c r="J32">
-        <v>3.2072743379244099E-44</v>
+        <v>3.6720657800608598E-7</v>
       </c>
       <c r="K32">
-        <v>2.3585121163045802E-34</v>
+        <v>5.9233812740040001E-6</v>
       </c>
       <c r="L32">
-        <v>8.7744278653098897E-26</v>
+        <v>6.8981334826136796E-5</v>
       </c>
       <c r="M32">
-        <v>1.6627822561720199E-18</v>
+        <v>5.8023053275164103E-4</v>
       </c>
       <c r="N32">
-        <v>1.6227502458287801E-12</v>
+        <v>3.5267438826822998E-3</v>
       </c>
       <c r="O32">
-        <v>8.3139721389703404E-8</v>
+        <v>1.54965636982205E-2</v>
       </c>
       <c r="P32">
-        <v>2.32159052392474E-4</v>
+        <v>4.9243458719037299E-2</v>
       </c>
       <c r="Q32">
-        <v>3.83538470474988E-2</v>
+        <v>0.11320090724259101</v>
       </c>
       <c r="R32">
-        <v>0.44776242294507301</v>
+        <v>0.18829682122989899</v>
       </c>
       <c r="S32">
-        <v>0.46898087312227299</v>
+        <v>0.22666962967252899</v>
       </c>
       <c r="T32">
-        <v>4.4371031965239803E-2</v>
+        <v>0.19748098318438401</v>
       </c>
       <c r="U32">
-        <v>2.9946257148227802E-4</v>
+        <v>0.124514725954384</v>
       </c>
       <c r="V32">
-        <v>1.20152062521583E-7</v>
+        <v>5.68093750930223E-2</v>
       </c>
       <c r="W32">
-        <v>2.6331159475034801E-12</v>
+        <v>1.8751023438100801E-2</v>
       </c>
       <c r="X32">
-        <v>0</v>
+        <v>4.4761389768565099E-3</v>
       </c>
       <c r="Y32">
-        <v>0</v>
+        <v>7.7249523484457401E-4</v>
       </c>
       <c r="Z32">
-        <v>0</v>
+        <v>9.6343072251037505E-5</v>
       </c>
       <c r="AA32">
-        <v>0</v>
+        <v>8.6792440920913298E-6</v>
       </c>
       <c r="AB32">
-        <v>0</v>
+        <v>5.6451607055585501E-7</v>
       </c>
       <c r="AC32">
-        <v>0</v>
+        <v>2.6497061544894599E-8</v>
       </c>
       <c r="AD32">
-        <v>0</v>
+        <v>8.9710383566199705E-10</v>
       </c>
       <c r="AE32">
-        <v>0</v>
+        <v>2.1898483026916499E-11</v>
       </c>
       <c r="AF32">
-        <v>0</v>
+        <v>3.8524738954492998E-13</v>
       </c>
       <c r="AG32">
-        <v>0</v>
+        <v>4.4408920985006404E-15</v>
       </c>
       <c r="AH32">
-        <v>0</v>
+        <v>4.44089209850064E-16</v>
       </c>
       <c r="AI32">
         <v>0</v>
@@ -87574,85 +87574,85 @@
         <v>11</v>
       </c>
       <c r="F33">
-        <v>7.5910278668329105E-147</v>
+        <v>2.2146980579714301E-17</v>
       </c>
       <c r="G33">
-        <v>1.3544843060758001E-124</v>
+        <v>4.7952790816832803E-15</v>
       </c>
       <c r="H33">
-        <v>3.3943658265632397E-104</v>
+        <v>6.7852659084208603E-13</v>
       </c>
       <c r="I33">
-        <v>1.19647941501129E-85</v>
+        <v>6.2788328499923303E-11</v>
       </c>
       <c r="J33">
-        <v>5.9439947585809098E-69</v>
+        <v>3.8026931594536901E-9</v>
       </c>
       <c r="K33">
-        <v>4.17312862300596E-54</v>
+        <v>1.50862115162799E-7</v>
       </c>
       <c r="L33">
-        <v>4.1565702546409299E-41</v>
+        <v>3.9242197058121998E-6</v>
       </c>
       <c r="M33">
-        <v>5.9073645354196499E-30</v>
+        <v>6.6995026337586698E-5</v>
       </c>
       <c r="N33">
-        <v>1.20884014861468E-20</v>
+        <v>7.5143696935234803E-4</v>
       </c>
       <c r="O33">
-        <v>3.6170967094169999E-13</v>
+        <v>5.5429938868736201E-3</v>
       </c>
       <c r="P33">
-        <v>1.62968810338509E-7</v>
+        <v>2.6916283873609798E-2</v>
       </c>
       <c r="Q33">
-        <v>1.18014743350423E-3</v>
+        <v>8.6114045896534E-2</v>
       </c>
       <c r="R33">
-        <v>0.16396731876158399</v>
+        <v>0.18164290701282801</v>
       </c>
       <c r="S33">
-        <v>0.69779131078025802</v>
+        <v>0.25272716997040001</v>
       </c>
       <c r="T33">
-        <v>0.13627426226741801</v>
+        <v>0.23198926002711501</v>
       </c>
       <c r="U33">
-        <v>7.8671206293035002E-4</v>
+        <v>0.14048885032632499</v>
       </c>
       <c r="V33">
-        <v>8.5724982668011696E-8</v>
+        <v>5.6109146615456601E-2</v>
       </c>
       <c r="W33">
-        <v>1.49324996812083E-13</v>
+        <v>1.47706223817302E-2</v>
       </c>
       <c r="X33">
-        <v>0</v>
+        <v>2.5609871029738098E-3</v>
       </c>
       <c r="Y33">
-        <v>0</v>
+        <v>2.9219146012249303E-4</v>
       </c>
       <c r="Z33">
-        <v>0</v>
+        <v>2.1915406008154999E-5</v>
       </c>
       <c r="AA33">
-        <v>0</v>
+        <v>1.07946505312206E-6</v>
       </c>
       <c r="AB33">
-        <v>0</v>
+        <v>3.4882180921513903E-8</v>
       </c>
       <c r="AC33">
-        <v>0</v>
+        <v>7.3877404194178098E-10</v>
       </c>
       <c r="AD33">
-        <v>0</v>
+        <v>1.0245582160450799E-11</v>
       </c>
       <c r="AE33">
-        <v>0</v>
+        <v>9.2925667161125602E-14</v>
       </c>
       <c r="AF33">
-        <v>0</v>
+        <v>5.5511151231257797E-16</v>
       </c>
       <c r="AG33">
         <v>0</v>
@@ -87942,91 +87942,91 @@
         <v>12</v>
       </c>
       <c r="F34">
-        <v>5.7265433313980999E-145</v>
+        <v>4.9979292827458596E-15</v>
       </c>
       <c r="G34">
-        <v>1.37732327244287E-123</v>
+        <v>4.17655407183452E-13</v>
       </c>
       <c r="H34">
-        <v>6.1848859515589397E-104</v>
+        <v>2.4912538567703699E-11</v>
       </c>
       <c r="I34">
-        <v>5.1924338148120403E-86</v>
+        <v>1.06115684133317E-9</v>
       </c>
       <c r="J34">
-        <v>8.1645397489471399E-70</v>
+        <v>3.2292779371551501E-8</v>
       </c>
       <c r="K34">
-        <v>2.4102750832462699E-55</v>
+        <v>7.0243907944404202E-7</v>
       </c>
       <c r="L34">
-        <v>1.3404436037461499E-42</v>
+        <v>1.0927225144842699E-5</v>
       </c>
       <c r="M34">
-        <v>1.4113212259303699E-31</v>
+        <v>1.21627793415456E-4</v>
       </c>
       <c r="N34">
-        <v>2.8346748370459901E-22</v>
+        <v>9.6916742857511902E-4</v>
       </c>
       <c r="O34">
-        <v>1.09984643502602E-14</v>
+        <v>5.5312105160696696E-3</v>
       </c>
       <c r="P34">
-        <v>8.4334423649434294E-9</v>
+        <v>2.2620016261007798E-2</v>
       </c>
       <c r="Q34">
-        <v>1.3398590477698699E-4</v>
+        <v>6.6311484387765393E-2</v>
       </c>
       <c r="R34">
-        <v>4.9598896285415403E-2</v>
+        <v>0.139395159824999</v>
       </c>
       <c r="S34">
-        <v>0.58692079552327003</v>
+        <v>0.210170262487339</v>
       </c>
       <c r="T34">
-        <v>0.35387113114768398</v>
+        <v>0.22730937835891099</v>
       </c>
       <c r="U34">
-        <v>9.4681706513143303E-3</v>
+        <v>0.176358809062543</v>
       </c>
       <c r="V34">
-        <v>7.0119395458867397E-6</v>
+        <v>9.8146448622744797E-2</v>
       </c>
       <c r="W34">
-        <v>1.14539377982225E-10</v>
+        <v>3.9171319382101298E-2</v>
       </c>
       <c r="X34">
-        <v>0</v>
+        <v>1.12087039181603E-2</v>
       </c>
       <c r="Y34">
-        <v>0</v>
+        <v>2.2986799336049998E-3</v>
       </c>
       <c r="Z34">
-        <v>0</v>
+        <v>3.3771629300838302E-4</v>
       </c>
       <c r="AA34">
-        <v>0</v>
+        <v>3.5527966892878697E-5</v>
       </c>
       <c r="AB34">
-        <v>0</v>
+        <v>2.6749493060584901E-6</v>
       </c>
       <c r="AC34">
-        <v>0</v>
+        <v>1.4406691639656799E-7</v>
       </c>
       <c r="AD34">
-        <v>0</v>
+        <v>5.5474550508805001E-9</v>
       </c>
       <c r="AE34">
-        <v>0</v>
+        <v>1.52646451034855E-10</v>
       </c>
       <c r="AF34">
-        <v>0</v>
+        <v>3.0001556794445601E-12</v>
       </c>
       <c r="AG34">
-        <v>0</v>
+        <v>3.8080649744642901E-14</v>
       </c>
       <c r="AH34">
-        <v>0</v>
+        <v>4.4408920985006301E-15</v>
       </c>
       <c r="AI34">
         <v>0</v>
@@ -88310,91 +88310,91 @@
         <v>13</v>
       </c>
       <c r="F35">
-        <v>3.8246036912444902E-73</v>
+        <v>2.4451499556567597E-13</v>
       </c>
       <c r="G35">
-        <v>1.0128492302328001E-62</v>
+        <v>1.04983651737671E-11</v>
       </c>
       <c r="H35">
-        <v>4.0466386012869399E-53</v>
+        <v>3.4148753959490699E-10</v>
       </c>
       <c r="I35">
-        <v>2.4421484216720899E-44</v>
+        <v>8.4175083167925193E-9</v>
       </c>
       <c r="J35">
-        <v>2.2298533303240299E-36</v>
+        <v>1.5727878668965799E-7</v>
       </c>
       <c r="K35">
-        <v>3.0870168287971899E-29</v>
+        <v>2.2282271422252999E-6</v>
       </c>
       <c r="L35">
-        <v>6.4989056068087603E-23</v>
+        <v>2.3942904978202499E-5</v>
       </c>
       <c r="M35">
-        <v>2.0893061852427499E-17</v>
+        <v>1.95184787299423E-4</v>
       </c>
       <c r="N35">
-        <v>1.03212573354446E-12</v>
+        <v>1.20749752136632E-3</v>
       </c>
       <c r="O35">
-        <v>7.9116733905037996E-9</v>
+        <v>5.6703521468957499E-3</v>
       </c>
       <c r="P35">
-        <v>9.5634742569771294E-6</v>
+        <v>2.0217135302555998E-2</v>
       </c>
       <c r="Q35">
-        <v>1.8744336212110301E-3</v>
+        <v>5.4739938938690703E-2</v>
       </c>
       <c r="R35">
-        <v>6.2465411897790403E-2</v>
+        <v>0.112573872640476</v>
       </c>
       <c r="S35">
-        <v>0.37936886689903598</v>
+        <v>0.17586311853561001</v>
       </c>
       <c r="T35">
-        <v>0.44808138071689302</v>
+        <v>0.20871366742299599</v>
       </c>
       <c r="U35">
-        <v>0.103724051497618</v>
+        <v>0.188182668649091</v>
       </c>
       <c r="V35">
-        <v>4.4434645638881101E-3</v>
+        <v>0.12889993542363601</v>
       </c>
       <c r="W35">
-        <v>3.2779888353040501E-5</v>
+        <v>6.7071840049615403E-2</v>
       </c>
       <c r="X35">
-        <v>3.9520697270312102E-8</v>
+        <v>2.6508902111763901E-2</v>
       </c>
       <c r="Y35">
-        <v>7.5478512329141203E-12</v>
+        <v>7.9567927047348493E-3</v>
       </c>
       <c r="Z35">
-        <v>2.2204460492503101E-16</v>
+        <v>1.8133994121650801E-3</v>
       </c>
       <c r="AA35">
-        <v>0</v>
+        <v>3.1373187921590698E-4</v>
       </c>
       <c r="AB35">
-        <v>0</v>
+        <v>4.1193001505513003E-5</v>
       </c>
       <c r="AC35">
-        <v>0</v>
+        <v>4.1036459874632796E-6</v>
       </c>
       <c r="AD35">
-        <v>0</v>
+        <v>3.1008098166918201E-7</v>
       </c>
       <c r="AE35">
-        <v>0</v>
+        <v>1.77669958745242E-8</v>
       </c>
       <c r="AF35">
-        <v>0</v>
+        <v>7.7172279677740004E-10</v>
       </c>
       <c r="AG35">
-        <v>0</v>
+        <v>2.18041140698234E-11</v>
       </c>
       <c r="AH35">
-        <v>0</v>
+        <v>4.2451597792592296E-12</v>
       </c>
       <c r="AI35">
         <v>0</v>
@@ -88678,91 +88678,91 @@
         <v>14</v>
       </c>
       <c r="F36">
-        <v>2.18164801345091E-26</v>
+        <v>1.93630267326368E-7</v>
       </c>
       <c r="G36">
-        <v>7.4811321873339602E-23</v>
+        <v>1.1318797927076999E-6</v>
       </c>
       <c r="H36">
-        <v>1.3763043924515199E-19</v>
+        <v>5.8457999847400001E-6</v>
       </c>
       <c r="I36">
-        <v>1.35950846668459E-16</v>
+        <v>2.6675560925485799E-5</v>
       </c>
       <c r="J36">
-        <v>7.2191341770498998E-14</v>
+        <v>1.07551894506716E-4</v>
       </c>
       <c r="K36">
-        <v>2.0637209630322701E-11</v>
+        <v>3.8314741301215602E-4</v>
       </c>
       <c r="L36">
-        <v>3.18154329117884E-9</v>
+        <v>1.2060489642207199E-3</v>
       </c>
       <c r="M36">
-        <v>2.6506525261577798E-7</v>
+        <v>3.35445888092565E-3</v>
       </c>
       <c r="N36">
-        <v>1.19635564291462E-5</v>
+        <v>8.2441356267943609E-3</v>
       </c>
       <c r="O36">
-        <v>2.9334111832386202E-4</v>
+        <v>1.7903537323554899E-2</v>
       </c>
       <c r="P36">
-        <v>3.91934421740149E-3</v>
+        <v>3.4356493672141303E-2</v>
       </c>
       <c r="Q36">
-        <v>2.8624469090622402E-2</v>
+        <v>5.82585313678112E-2</v>
       </c>
       <c r="R36">
-        <v>0.11460805792574801</v>
+        <v>8.7296046967528004E-2</v>
       </c>
       <c r="S36">
-        <v>0.25216375665083401</v>
+        <v>0.115589073749297</v>
       </c>
       <c r="T36">
-        <v>0.30534743392022301</v>
+        <v>0.13524714770355301</v>
       </c>
       <c r="U36">
-        <v>0.20357135716980199</v>
+        <v>0.13983943996912501</v>
       </c>
       <c r="V36">
-        <v>7.4662144488841606E-2</v>
+        <v>0.12776788403188299</v>
       </c>
       <c r="W36">
-        <v>1.5036236279628501E-2</v>
+        <v>0.10315815319752</v>
       </c>
       <c r="X36">
-        <v>1.65842112212954E-3</v>
+        <v>7.3599309895679296E-2</v>
       </c>
       <c r="Y36">
-        <v>9.9873597110389193E-5</v>
+        <v>4.6401273098600197E-2</v>
       </c>
       <c r="Z36">
-        <v>3.2737936974669398E-6</v>
+        <v>2.5850492743526101E-2</v>
       </c>
       <c r="AA36">
-        <v>5.8238046829472899E-8</v>
+        <v>1.27258418022775E-2</v>
       </c>
       <c r="AB36">
-        <v>5.6073157228553296E-10</v>
+        <v>5.5357718500575297E-3</v>
       </c>
       <c r="AC36">
-        <v>2.9153346403631901E-12</v>
+        <v>2.12783655078612E-3</v>
       </c>
       <c r="AD36">
-        <v>8.2156503822261505E-15</v>
+        <v>7.2270407169187402E-4</v>
       </c>
       <c r="AE36">
-        <v>0</v>
+        <v>2.1688921516100501E-4</v>
       </c>
       <c r="AF36">
-        <v>0</v>
+        <v>5.7512608931914503E-5</v>
       </c>
       <c r="AG36">
-        <v>0</v>
+        <v>9.1876580897446606E-6</v>
       </c>
       <c r="AH36">
-        <v>0</v>
+        <v>7.6828723546611304E-6</v>
       </c>
       <c r="AI36">
         <v>0</v>
@@ -89046,85 +89046,85 @@
         <v>15</v>
       </c>
       <c r="F37">
-        <v>6.6212494678606005E-79</v>
+        <v>3.87172912891438E-24</v>
       </c>
       <c r="G37">
-        <v>5.9563542175959802E-68</v>
+        <v>4.6015374904078402E-21</v>
       </c>
       <c r="H37">
-        <v>7.7832342894770701E-58</v>
+        <v>3.2645812226302801E-18</v>
       </c>
       <c r="I37">
-        <v>1.4789939827070699E-48</v>
+        <v>1.38359135192944E-15</v>
       </c>
       <c r="J37">
-        <v>4.0928787932895603E-40</v>
+        <v>3.50615509437634E-13</v>
       </c>
       <c r="K37">
-        <v>1.65264248036615E-32</v>
+        <v>5.3180206041090798E-11</v>
       </c>
       <c r="L37">
-        <v>9.7621424169533605E-26</v>
+        <v>4.8338072221461299E-9</v>
       </c>
       <c r="M37">
-        <v>8.4666452521495795E-20</v>
+        <v>2.6366309665085999E-7</v>
       </c>
       <c r="N37">
-        <v>1.08390571600307E-14</v>
+        <v>8.6437764801977597E-6</v>
       </c>
       <c r="O37">
-        <v>2.0650729604495099E-10</v>
+        <v>1.7060327081592499E-4</v>
       </c>
       <c r="P37">
-        <v>5.9334125531472096E-7</v>
+        <v>2.03083833574825E-3</v>
       </c>
       <c r="Q37">
-        <v>2.6300916593789898E-4</v>
+        <v>1.4606430641634501E-2</v>
       </c>
       <c r="R37">
-        <v>1.87158408212106E-2</v>
+        <v>6.3580159647888906E-2</v>
       </c>
       <c r="S37">
-        <v>0.22798985729420601</v>
+        <v>0.16773644013028299</v>
       </c>
       <c r="T37">
-        <v>0.51330419282764395</v>
+        <v>0.26848000659577398</v>
       </c>
       <c r="U37">
-        <v>0.22179261298153399</v>
+        <v>0.26085962991158901</v>
       </c>
       <c r="V37">
-        <v>1.7692078895811699E-2</v>
+        <v>0.153850088284264</v>
       </c>
       <c r="W37">
-        <v>2.41286462937417E-4</v>
+        <v>5.5045998916998101E-2</v>
       </c>
       <c r="X37">
-        <v>5.2782488946245799E-7</v>
+        <v>1.19348813632386E-2</v>
       </c>
       <c r="Y37">
-        <v>1.7804524521380901E-10</v>
+        <v>1.5658118379778801E-3</v>
       </c>
       <c r="Z37">
-        <v>9.1038288019262805E-15</v>
+        <v>1.2409480235919801E-4</v>
       </c>
       <c r="AA37">
-        <v>0</v>
+        <v>5.9303657836684598E-6</v>
       </c>
       <c r="AB37">
-        <v>0</v>
+        <v>1.7058922796575599E-7</v>
       </c>
       <c r="AC37">
-        <v>0</v>
+        <v>2.9487279284978699E-9</v>
       </c>
       <c r="AD37">
-        <v>0</v>
+        <v>3.0581981391719598E-11</v>
       </c>
       <c r="AE37">
-        <v>0</v>
+        <v>1.90070181815827E-13</v>
       </c>
       <c r="AF37">
-        <v>0</v>
+        <v>6.6613381477509402E-16</v>
       </c>
       <c r="AG37">
         <v>0</v>
@@ -89414,79 +89414,79 @@
         <v>16</v>
       </c>
       <c r="F38">
-        <v>7.4558822853686197E-77</v>
+        <v>2.1642875271851701E-38</v>
       </c>
       <c r="G38">
-        <v>2.7133555296763898E-66</v>
+        <v>1.6866738608362901E-33</v>
       </c>
       <c r="H38">
-        <v>1.5671249665017599E-56</v>
+        <v>5.89266157944381E-29</v>
       </c>
       <c r="I38">
-        <v>1.4380067134866201E-47</v>
+        <v>9.2369707773373906E-25</v>
       </c>
       <c r="J38">
-        <v>2.0993490628977801E-39</v>
+        <v>6.5035549558178998E-21</v>
       </c>
       <c r="K38">
-        <v>4.8850876035913902E-32</v>
+        <v>2.0595007246728901E-17</v>
       </c>
       <c r="L38">
-        <v>1.81635898862387E-25</v>
+        <v>2.9383920578321999E-14</v>
       </c>
       <c r="M38">
-        <v>1.08286981346921E-19</v>
+        <v>1.89300266207815E-11</v>
       </c>
       <c r="N38">
-        <v>1.0403431139236701E-14</v>
+        <v>5.5222381212390703E-9</v>
       </c>
       <c r="O38">
-        <v>1.6229865073183901E-10</v>
+        <v>7.3209814929611701E-7</v>
       </c>
       <c r="P38">
-        <v>4.16191245164241E-7</v>
+        <v>4.4307630964427802E-5</v>
       </c>
       <c r="Q38">
-        <v>1.79069947822913E-4</v>
+        <v>1.2308923776336699E-3</v>
       </c>
       <c r="R38">
-        <v>1.33889448722622E-2</v>
+        <v>1.5794477528508599E-2</v>
       </c>
       <c r="S38">
-        <v>0.18394280661123</v>
+        <v>9.42212840681909E-2</v>
       </c>
       <c r="T38">
-        <v>0.496921487898279</v>
+        <v>0.26282472357019998</v>
       </c>
       <c r="U38">
-        <v>0.27464814463149201</v>
+        <v>0.34416599281702198</v>
       </c>
       <c r="V38">
-        <v>3.0292455023614599E-2</v>
+        <v>0.21180785767591301</v>
       </c>
       <c r="W38">
-        <v>6.2440963266319205E-4</v>
+        <v>6.1139547051804702E-2</v>
       </c>
       <c r="X38">
-        <v>2.2636421542765402E-6</v>
+        <v>8.2398047377154598E-3</v>
       </c>
       <c r="Y38">
-        <v>1.3867857973082199E-9</v>
+        <v>5.1531871330279299E-4</v>
       </c>
       <c r="Z38">
-        <v>1.4022116801015699E-13</v>
+        <v>1.4858668772155201E-5</v>
       </c>
       <c r="AA38">
-        <v>0</v>
+        <v>1.9633471237678901E-7</v>
       </c>
       <c r="AB38">
-        <v>0</v>
+        <v>1.18267473592226E-9</v>
       </c>
       <c r="AC38">
-        <v>0</v>
+        <v>3.2339686484306201E-12</v>
       </c>
       <c r="AD38">
-        <v>0</v>
+        <v>3.9968028886505604E-15</v>
       </c>
       <c r="AE38">
         <v>0</v>
@@ -89782,91 +89782,91 @@
         <v>17</v>
       </c>
       <c r="F39">
-        <v>1.7984134793164E-115</v>
+        <v>1.4008003911826199E-19</v>
       </c>
       <c r="G39">
-        <v>1.3976336806378501E-99</v>
+        <v>3.3044476005478799E-17</v>
       </c>
       <c r="H39">
-        <v>6.9187522253910702E-85</v>
+        <v>5.3140973483567402E-15</v>
       </c>
       <c r="I39">
-        <v>2.1840299434735901E-71</v>
+        <v>5.8288579753187203E-13</v>
       </c>
       <c r="J39">
-        <v>4.4023572677444904E-59</v>
+        <v>4.36314348053882E-11</v>
       </c>
       <c r="K39">
-        <v>5.6767172746568505E-48</v>
+        <v>2.2301790514753601E-9</v>
       </c>
       <c r="L39">
-        <v>4.69421201430927E-38</v>
+        <v>7.7891228766818304E-8</v>
       </c>
       <c r="M39">
-        <v>2.4979030795077301E-29</v>
+        <v>1.8601571131258199E-6</v>
       </c>
       <c r="N39">
-        <v>8.5963234112908499E-22</v>
+        <v>3.0397712291622298E-5</v>
       </c>
       <c r="O39">
-        <v>1.9280322861589801E-15</v>
+        <v>3.4016310196174199E-4</v>
       </c>
       <c r="P39">
-        <v>2.8540352057500698E-10</v>
+        <v>2.6086170031895E-3</v>
       </c>
       <c r="Q39">
-        <v>2.8520046547842599E-6</v>
+        <v>1.37188203741363E-2</v>
       </c>
       <c r="R39">
-        <v>2.0120507598861601E-3</v>
+        <v>4.9508972184522999E-2</v>
       </c>
       <c r="S39">
-        <v>0.110247251568836</v>
+        <v>0.12267200592882301</v>
       </c>
       <c r="T39">
-        <v>0.56017342511012902</v>
+        <v>0.20877471851712601</v>
       </c>
       <c r="U39">
-        <v>0.31004383692811399</v>
+        <v>0.24411209166584799</v>
       </c>
       <c r="V39">
-        <v>1.7438670028366899E-2</v>
+        <v>0.19611557372923499</v>
       </c>
       <c r="W39">
-        <v>8.1885192785735502E-5</v>
+        <v>0.10824327456011799</v>
       </c>
       <c r="X39">
-        <v>2.8121157513716299E-8</v>
+        <v>4.1033231882233998E-2</v>
       </c>
       <c r="Y39">
-        <v>6.6291416800368097E-13</v>
+        <v>1.06789762083551E-2</v>
       </c>
       <c r="Z39">
-        <v>0</v>
+        <v>1.9069557683903901E-3</v>
       </c>
       <c r="AA39">
-        <v>0</v>
+        <v>2.3349925616567E-4</v>
       </c>
       <c r="AB39">
-        <v>0</v>
+        <v>1.95908947671075E-5</v>
       </c>
       <c r="AC39">
-        <v>0</v>
+        <v>1.1254438880836699E-6</v>
       </c>
       <c r="AD39">
-        <v>0</v>
+        <v>4.4235396234881799E-8</v>
       </c>
       <c r="AE39">
-        <v>0</v>
+        <v>1.1887115736186601E-9</v>
       </c>
       <c r="AF39">
-        <v>0</v>
+        <v>2.1824431151173901E-11</v>
       </c>
       <c r="AG39">
-        <v>0</v>
+        <v>2.4913404672588498E-13</v>
       </c>
       <c r="AH39">
-        <v>0</v>
+        <v>2.6756374893466301E-14</v>
       </c>
       <c r="AI39">
         <v>0</v>
@@ -90150,91 +90150,91 @@
         <v>18</v>
       </c>
       <c r="F40">
-        <v>1.5435350339625601E-64</v>
+        <v>2.00032129667094E-13</v>
       </c>
       <c r="G40">
-        <v>7.9072699057265698E-56</v>
+        <v>5.0431915002124603E-12</v>
       </c>
       <c r="H40">
-        <v>9.08625853932987E-48</v>
+        <v>1.03919872297257E-10</v>
       </c>
       <c r="I40">
-        <v>2.3444344715632201E-40</v>
+        <v>1.75035774300499E-9</v>
       </c>
       <c r="J40">
-        <v>1.3600543542888399E-33</v>
+        <v>2.41011709124361E-8</v>
       </c>
       <c r="K40">
-        <v>1.7769916342409199E-27</v>
+        <v>2.7131924986071899E-7</v>
       </c>
       <c r="L40">
-        <v>5.2411255402672003E-22</v>
+        <v>2.4974786758218799E-6</v>
       </c>
       <c r="M40">
-        <v>3.50067394234254E-17</v>
+        <v>1.8799585958294798E-5</v>
       </c>
       <c r="N40">
-        <v>5.3190168117315404E-13</v>
+        <v>1.15735119692212E-4</v>
       </c>
       <c r="O40">
-        <v>1.8508405852857101E-9</v>
+        <v>5.82767586028286E-4</v>
       </c>
       <c r="P40">
-        <v>1.49008750473707E-6</v>
+        <v>2.4003755478933502E-3</v>
       </c>
       <c r="Q40">
-        <v>2.8203768462971599E-4</v>
+        <v>8.0882301846764496E-3</v>
       </c>
       <c r="R40">
-        <v>1.28624236802167E-2</v>
+        <v>2.22972508576477E-2</v>
       </c>
       <c r="S40">
-        <v>0.146273708251762</v>
+        <v>5.0292263810199203E-2</v>
       </c>
       <c r="T40">
-        <v>0.43082756563643299</v>
+        <v>9.2816815752497006E-2</v>
       </c>
       <c r="U40">
-        <v>0.33666974574338898</v>
+        <v>0.140167047953728</v>
       </c>
       <c r="V40">
-        <v>6.9382460310257799E-2</v>
+        <v>0.17320937509988801</v>
       </c>
       <c r="W40">
-        <v>3.6531142358710001E-3</v>
+        <v>0.17514974699555999</v>
       </c>
       <c r="X40">
-        <v>4.7306324449936099E-5</v>
+        <v>0.144930778684419</v>
       </c>
       <c r="Y40">
-        <v>1.4608875054111699E-7</v>
+        <v>9.81338772150286E-2</v>
       </c>
       <c r="Z40">
-        <v>1.0534406680306999E-10</v>
+        <v>5.4371678622098997E-2</v>
       </c>
       <c r="AA40">
-        <v>1.7541523789077401E-14</v>
+        <v>2.4649290994365702E-2</v>
       </c>
       <c r="AB40">
-        <v>0</v>
+        <v>9.1430489030997503E-3</v>
       </c>
       <c r="AC40">
-        <v>0</v>
+        <v>2.7746267178104999E-3</v>
       </c>
       <c r="AD40">
-        <v>0</v>
+        <v>6.8883064294656304E-4</v>
       </c>
       <c r="AE40">
-        <v>0</v>
+        <v>1.3988727614744399E-4</v>
       </c>
       <c r="AF40">
-        <v>0</v>
+        <v>2.3236029949247501E-5</v>
       </c>
       <c r="AG40">
-        <v>0</v>
+        <v>2.3448187761454702E-6</v>
       </c>
       <c r="AH40">
-        <v>0</v>
+        <v>1.1968429723951999E-6</v>
       </c>
       <c r="AI40">
         <v>0</v>
@@ -90518,82 +90518,82 @@
         <v>19</v>
       </c>
       <c r="F41">
-        <v>8.4607694781919796E-39</v>
+        <v>1.1388796001486E-38</v>
       </c>
       <c r="G41">
-        <v>1.09127882779661E-33</v>
+        <v>5.5957517607714699E-34</v>
       </c>
       <c r="H41">
-        <v>5.9072606033327405E-29</v>
+        <v>1.32514015656734E-29</v>
       </c>
       <c r="I41">
-        <v>1.34332153606179E-24</v>
+        <v>1.5135667452032199E-25</v>
       </c>
       <c r="J41">
-        <v>1.2848341783522999E-20</v>
+        <v>8.34570334340603E-22</v>
       </c>
       <c r="K41">
-        <v>5.1768333954738598E-17</v>
+        <v>2.2239412568061799E-18</v>
       </c>
       <c r="L41">
-        <v>8.8045319496828604E-14</v>
+        <v>2.8679979163494298E-15</v>
       </c>
       <c r="M41">
-        <v>6.3374570585598506E-11</v>
+        <v>1.7929892901601301E-12</v>
       </c>
       <c r="N41">
-        <v>1.9372493389080599E-8</v>
+        <v>5.4457756078265998E-10</v>
       </c>
       <c r="O41">
-        <v>2.52618019742128E-6</v>
+        <v>8.0574795838780401E-8</v>
       </c>
       <c r="P41">
-        <v>1.41330285132979E-4</v>
+        <v>5.8269635969887796E-6</v>
       </c>
       <c r="Q41">
-        <v>3.41616421208736E-3</v>
+        <v>2.0678687980087401E-4</v>
       </c>
       <c r="R41">
-        <v>3.5961432504904703E-2</v>
+        <v>3.6176856030226199E-3</v>
       </c>
       <c r="S41">
-        <v>0.166199862877839</v>
+        <v>3.1354451737305902E-2</v>
       </c>
       <c r="T41">
-        <v>0.33948193460927301</v>
+        <v>0.13526707565917001</v>
       </c>
       <c r="U41">
-        <v>0.30758340925994099</v>
+        <v>0.29161094796968101</v>
       </c>
       <c r="V41">
-        <v>0.123550207466033</v>
+        <v>0.31487872020561197</v>
       </c>
       <c r="W41">
-        <v>2.1903260262320801E-2</v>
+        <v>0.17033991497057899</v>
       </c>
       <c r="X41">
-        <v>1.70155768950208E-3</v>
+        <v>4.6078873302335503E-2</v>
       </c>
       <c r="Y41">
-        <v>5.7453359196601899E-5</v>
+        <v>6.2105752545303901E-3</v>
       </c>
       <c r="Z41">
-        <v>8.3662478411738995E-7</v>
+        <v>4.1514185191893199E-4</v>
       </c>
       <c r="AA41">
-        <v>5.2189425003845696E-9</v>
+        <v>1.3694806267006099E-5</v>
       </c>
       <c r="AB41">
-        <v>1.3871459536574E-11</v>
+        <v>2.2190922877030101E-7</v>
       </c>
       <c r="AC41">
-        <v>1.5654144647214701E-14</v>
+        <v>1.7589726342137601E-9</v>
       </c>
       <c r="AD41">
-        <v>0</v>
+        <v>6.7966743344527499E-12</v>
       </c>
       <c r="AE41">
-        <v>0</v>
+        <v>1.27675647831893E-14</v>
       </c>
       <c r="AF41">
         <v>0</v>
@@ -90886,88 +90886,88 @@
         <v>20</v>
       </c>
       <c r="F42">
-        <v>2.1130876209901901E-57</v>
+        <v>1.5824356892955E-24</v>
       </c>
       <c r="G42">
-        <v>9.5610015750838797E-50</v>
+        <v>1.66532987780435E-21</v>
       </c>
       <c r="H42">
-        <v>1.1774779543405801E-42</v>
+        <v>1.07489476294313E-18</v>
       </c>
       <c r="I42">
-        <v>3.95090419610033E-36</v>
+        <v>4.2580648469235702E-16</v>
       </c>
       <c r="J42">
-        <v>3.6164603378182202E-30</v>
+        <v>1.03603907272714E-13</v>
       </c>
       <c r="K42">
-        <v>9.0454196730779299E-25</v>
+        <v>1.5497016302162099E-11</v>
       </c>
       <c r="L42">
-        <v>6.1955859315874001E-20</v>
+        <v>1.42651790033228E-9</v>
       </c>
       <c r="M42">
-        <v>1.1655847474977699E-15</v>
+        <v>8.0904682607325396E-8</v>
       </c>
       <c r="N42">
-        <v>6.0483794944594904E-12</v>
+        <v>2.8307850178286801E-6</v>
       </c>
       <c r="O42">
-        <v>8.7097569831647902E-9</v>
+        <v>6.1192456245726901E-5</v>
       </c>
       <c r="P42">
-        <v>3.5118575609102E-6</v>
+        <v>8.1846993400162805E-4</v>
       </c>
       <c r="Q42">
-        <v>4.0177949103648399E-4</v>
+        <v>6.7840055347346898E-3</v>
       </c>
       <c r="R42">
-        <v>1.3291660212459099E-2</v>
+        <v>3.4896761916008101E-2</v>
       </c>
       <c r="S42">
-        <v>0.13029220663635899</v>
+        <v>0.11154855294013399</v>
       </c>
       <c r="T42">
-        <v>0.38818019591278202</v>
+        <v>0.22180292110998101</v>
       </c>
       <c r="U42">
-        <v>0.35735744634861399</v>
+        <v>0.2745222048898</v>
       </c>
       <c r="V42">
-        <v>0.101514153936898</v>
+        <v>0.21153651514784599</v>
       </c>
       <c r="W42">
-        <v>8.7354869436807592E-3</v>
+        <v>0.101456563109974</v>
       </c>
       <c r="X42">
-        <v>2.21921286363557E-4</v>
+        <v>3.02664629337152E-2</v>
       </c>
       <c r="Y42">
-        <v>1.6252864845078799E-6</v>
+        <v>5.6101083217721098E-3</v>
       </c>
       <c r="Z42">
-        <v>3.36999872452281E-9</v>
+        <v>6.4526052007396505E-4</v>
       </c>
       <c r="AA42">
-        <v>1.9536594564328799E-12</v>
+        <v>4.5984520293140798E-5</v>
       </c>
       <c r="AB42">
-        <v>3.3306690738754598E-16</v>
+        <v>2.0273818590599299E-6</v>
       </c>
       <c r="AC42">
-        <v>0</v>
+        <v>5.5214506855527599E-8</v>
       </c>
       <c r="AD42">
-        <v>0</v>
+        <v>9.2757312941671402E-10</v>
       </c>
       <c r="AE42">
-        <v>0</v>
+        <v>9.5996544047238802E-12</v>
       </c>
       <c r="AF42">
-        <v>0</v>
+        <v>6.11732886568461E-14</v>
       </c>
       <c r="AG42">
-        <v>0</v>
+        <v>2.2204460492503101E-16</v>
       </c>
       <c r="AH42">
         <v>0</v>
@@ -91254,76 +91254,76 @@
         <v>21</v>
       </c>
       <c r="F43">
-        <v>1.54922752988334E-44</v>
+        <v>2.2695885625866099E-67</v>
       </c>
       <c r="G43">
-        <v>1.1387488092960701E-38</v>
+        <v>3.3589233012317301E-59</v>
       </c>
       <c r="H43">
-        <v>3.1051154149926301E-33</v>
+        <v>1.4256145792938701E-51</v>
       </c>
       <c r="I43">
-        <v>3.1440025998520298E-28</v>
+        <v>1.73644199613014E-44</v>
       </c>
       <c r="J43">
-        <v>1.1835141991984699E-23</v>
+        <v>6.0751336716625703E-38</v>
       </c>
       <c r="K43">
-        <v>1.6589459856459901E-19</v>
+        <v>6.1118129671422101E-32</v>
       </c>
       <c r="L43">
-        <v>8.6766867355623495E-16</v>
+        <v>1.77060510257876E-26</v>
       </c>
       <c r="M43">
-        <v>1.6979710411868301E-12</v>
+        <v>1.47986946350836E-21</v>
       </c>
       <c r="N43">
-        <v>1.2478712883246701E-9</v>
+        <v>3.5774042515175797E-17</v>
       </c>
       <c r="O43">
-        <v>3.4614333802514299E-7</v>
+        <v>2.5099435167595401E-13</v>
       </c>
       <c r="P43">
-        <v>3.6486416110942201E-5</v>
+        <v>5.1362729230524498E-10</v>
       </c>
       <c r="Q43">
-        <v>1.4745073402478001E-3</v>
+        <v>3.0875498121532199E-7</v>
       </c>
       <c r="R43">
-        <v>2.3096127106089201E-2</v>
+        <v>5.5090781258938899E-5</v>
       </c>
       <c r="S43">
-        <v>0.14190772045219399</v>
+        <v>2.9615402582734E-3</v>
       </c>
       <c r="T43">
-        <v>0.34571799418282201</v>
+        <v>4.8933102340906497E-2</v>
       </c>
       <c r="U43">
-        <v>0.33611289043322301</v>
+        <v>0.25429170998919898</v>
       </c>
       <c r="V43">
-        <v>0.130376996076741</v>
+        <v>0.42387622602463298</v>
       </c>
       <c r="W43">
-        <v>2.0040977669610101E-2</v>
+        <v>0.22832274776022901</v>
       </c>
       <c r="X43">
-        <v>1.2075204616538401E-3</v>
+        <v>3.9390929337003402E-2</v>
       </c>
       <c r="Y43">
-        <v>2.8179639063097199E-5</v>
+        <v>2.1327493867024901E-3</v>
       </c>
       <c r="Z43">
-        <v>2.5197247344177498E-7</v>
+        <v>3.5417677128224398E-5</v>
       </c>
       <c r="AA43">
-        <v>8.55763904183959E-10</v>
+        <v>1.7691369613714901E-7</v>
       </c>
       <c r="AB43">
-        <v>1.09656728142226E-12</v>
+        <v>2.61996424555377E-10</v>
       </c>
       <c r="AC43">
-        <v>5.5511151231257797E-16</v>
+        <v>1.1390888232654101E-13</v>
       </c>
       <c r="AD43">
         <v>0</v>

</xml_diff>